<commit_message>
Recalcula sem usar divisa; remove coluna Situação do CSV exportado
Pipeline agora só usa estrada desenhada pro cálculo de distância — divisa de
talhão nunca mais entra, nem como último recurso (antes era só penalizada
1000x). 60 dos 351 talhões ficaram sem estrada mapeada até eles e aparecem
como "sem estrada mapeada até este talhão" em vez de uma distância inventada
pela divisa; lista completa em talhoes_sem_estrada.csv no repositório do
pipeline. Tucano concentra a maioria (35 de 70) por ser a fazenda com menos
estrada desenhada.

Também remove a coluna "Situação" dos três tipos de exportação CSV do site,
a pedido.
</commit_message>
<xml_diff>
--- a/FAZENDA_JAVA_distancias.xlsx
+++ b/FAZENDA_JAVA_distancias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\talhao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2675BE48-6499-43C4-8541-893665717D17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BBA2AD1-FAC8-43C4-849A-42B1D6480D99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1884" yWindow="1884" windowWidth="14100" windowHeight="9792" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Distâncias" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="73">
   <si>
     <t>FAZENDA JAVA — distância dos talhões até a sede</t>
   </si>
@@ -72,109 +72,118 @@
     <t>Observação</t>
   </si>
   <si>
+    <t>T-11B</t>
+  </si>
+  <si>
+    <t>T-11C</t>
+  </si>
+  <si>
     <t>T-11A</t>
   </si>
   <si>
+    <t>T-11D</t>
+  </si>
+  <si>
+    <t>T-13A</t>
+  </si>
+  <si>
+    <t>T-13B</t>
+  </si>
+  <si>
+    <t>T-13C</t>
+  </si>
+  <si>
     <t>T-13D</t>
   </si>
   <si>
-    <t>T-13C</t>
-  </si>
-  <si>
     <t>T-10A</t>
   </si>
   <si>
-    <t>T-11B</t>
-  </si>
-  <si>
-    <t>T-13B</t>
-  </si>
-  <si>
-    <t>T-11D</t>
-  </si>
-  <si>
     <t>T-12A</t>
   </si>
   <si>
-    <t>T-11C</t>
-  </si>
-  <si>
-    <t>T-13A</t>
+    <t>T-07A</t>
+  </si>
+  <si>
+    <t>T-09A</t>
+  </si>
+  <si>
+    <t>T-07B</t>
+  </si>
+  <si>
+    <t>T-14A</t>
+  </si>
+  <si>
+    <t>T-14D</t>
+  </si>
+  <si>
+    <t>T-15B</t>
+  </si>
+  <si>
+    <t>T-07D</t>
+  </si>
+  <si>
+    <t>T-07C</t>
+  </si>
+  <si>
+    <t>T-15C</t>
+  </si>
+  <si>
+    <t>T-05</t>
+  </si>
+  <si>
+    <t>T-01C</t>
+  </si>
+  <si>
+    <t>T-06B</t>
+  </si>
+  <si>
+    <t>T-06D</t>
+  </si>
+  <si>
+    <t>T-06E</t>
+  </si>
+  <si>
+    <t>T-06C</t>
+  </si>
+  <si>
+    <t>T-03B</t>
+  </si>
+  <si>
+    <t>T-03A</t>
+  </si>
+  <si>
+    <t>T-08A</t>
+  </si>
+  <si>
+    <t>T-01</t>
+  </si>
+  <si>
+    <t>T-04A</t>
+  </si>
+  <si>
+    <t>T-04B</t>
+  </si>
+  <si>
+    <t>T-01A</t>
+  </si>
+  <si>
+    <t>T-04</t>
+  </si>
+  <si>
+    <t>T-02</t>
   </si>
   <si>
     <t>T-09B</t>
   </si>
   <si>
-    <t>T-09A</t>
-  </si>
-  <si>
-    <t>T-15B</t>
-  </si>
-  <si>
-    <t>T-07B</t>
-  </si>
-  <si>
-    <t>T-08A</t>
-  </si>
-  <si>
-    <t>T-14A</t>
-  </si>
-  <si>
-    <t>T-14D</t>
-  </si>
-  <si>
-    <t>T-07A</t>
-  </si>
-  <si>
-    <t>T-07C</t>
-  </si>
-  <si>
-    <t>T-05</t>
-  </si>
-  <si>
-    <t>T-15C</t>
-  </si>
-  <si>
-    <t>T-07D</t>
-  </si>
-  <si>
-    <t>T-01C</t>
-  </si>
-  <si>
-    <t>T-03A</t>
-  </si>
-  <si>
-    <t>T-06C</t>
-  </si>
-  <si>
-    <t>T-06D</t>
-  </si>
-  <si>
-    <t>T-06B</t>
-  </si>
-  <si>
-    <t>T-06E</t>
-  </si>
-  <si>
-    <t>T-03B</t>
-  </si>
-  <si>
-    <t>T-04B</t>
-  </si>
-  <si>
-    <t>T-04A</t>
-  </si>
-  <si>
-    <t>T-01A</t>
-  </si>
-  <si>
-    <t>T-01</t>
-  </si>
-  <si>
-    <t>T-02</t>
-  </si>
-  <si>
-    <t>T-04</t>
+    <t>sem acesso</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>sem estrada até este talhão</t>
   </si>
   <si>
     <t>TOTAL / MÁXIMO</t>
@@ -253,7 +262,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -299,6 +308,17 @@
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FFC00000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FFC00000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF808080"/>
@@ -310,7 +330,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -325,6 +345,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -349,7 +374,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -370,13 +395,25 @@
     <xf numFmtId="4" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -745,31 +782,31 @@
         <v>12</v>
       </c>
       <c r="B5" s="5">
-        <v>61.24</v>
+        <v>46.69</v>
       </c>
       <c r="C5" s="6">
-        <v>3271</v>
+        <v>3078</v>
       </c>
       <c r="D5" s="7">
-        <v>26692</v>
+        <v>23878</v>
       </c>
       <c r="E5" s="7">
-        <v>22261</v>
+        <v>23285</v>
       </c>
       <c r="F5" s="7">
-        <v>11475</v>
+        <v>11323</v>
       </c>
       <c r="G5" s="8">
-        <f t="shared" ref="G5:G39" si="0">D5/1000</f>
-        <v>26.692</v>
+        <f t="shared" ref="G5:G38" si="0">D5/1000</f>
+        <v>23.878</v>
       </c>
       <c r="H5" s="8">
-        <f t="shared" ref="H5:H39" si="1">E5/1000</f>
-        <v>22.260999999999999</v>
+        <f t="shared" ref="H5:H38" si="1">E5/1000</f>
+        <v>23.285</v>
       </c>
       <c r="I5" s="9">
-        <f t="shared" ref="I5:I39" si="2">IFERROR(D5/F5,"")</f>
-        <v>2.3261002178649237</v>
+        <f t="shared" ref="I5:I38" si="2">IFERROR(D5/F5,"")</f>
+        <v>2.1088050869910799</v>
       </c>
       <c r="J5" s="10"/>
     </row>
@@ -778,31 +815,31 @@
         <v>13</v>
       </c>
       <c r="B6" s="12">
-        <v>61.56</v>
+        <v>52.01</v>
       </c>
       <c r="C6" s="13">
-        <v>3161</v>
+        <v>3100</v>
       </c>
       <c r="D6" s="14">
-        <v>26690</v>
+        <v>23878</v>
       </c>
       <c r="E6" s="14">
-        <v>22258</v>
+        <v>23285</v>
       </c>
       <c r="F6" s="14">
-        <v>11726</v>
+        <v>10871</v>
       </c>
       <c r="G6" s="15">
         <f t="shared" si="0"/>
-        <v>26.69</v>
+        <v>23.878</v>
       </c>
       <c r="H6" s="15">
         <f t="shared" si="1"/>
-        <v>22.257999999999999</v>
+        <v>23.285</v>
       </c>
       <c r="I6" s="16">
         <f t="shared" si="2"/>
-        <v>2.2761384956506907</v>
+        <v>2.1964860638395733</v>
       </c>
       <c r="J6" s="17"/>
     </row>
@@ -811,31 +848,31 @@
         <v>14</v>
       </c>
       <c r="B7" s="5">
-        <v>54.2</v>
+        <v>61.24</v>
       </c>
       <c r="C7" s="6">
-        <v>2992</v>
+        <v>3271</v>
       </c>
       <c r="D7" s="7">
-        <v>26326</v>
+        <v>23316</v>
       </c>
       <c r="E7" s="7">
-        <v>23076</v>
+        <v>22217</v>
       </c>
       <c r="F7" s="7">
-        <v>11982</v>
+        <v>11475</v>
       </c>
       <c r="G7" s="8">
         <f t="shared" si="0"/>
-        <v>26.326000000000001</v>
+        <v>23.315999999999999</v>
       </c>
       <c r="H7" s="8">
         <f t="shared" si="1"/>
-        <v>23.076000000000001</v>
+        <v>22.216999999999999</v>
       </c>
       <c r="I7" s="9">
         <f t="shared" si="2"/>
-        <v>2.1971290268736436</v>
+        <v>2.0318954248366015</v>
       </c>
       <c r="J7" s="10"/>
     </row>
@@ -844,31 +881,31 @@
         <v>15</v>
       </c>
       <c r="B8" s="12">
-        <v>67.819999999999993</v>
+        <v>70.47</v>
       </c>
       <c r="C8" s="13">
-        <v>4140</v>
+        <v>3481</v>
       </c>
       <c r="D8" s="14">
-        <v>25609</v>
+        <v>23316</v>
       </c>
       <c r="E8" s="14">
-        <v>20476</v>
+        <v>21484</v>
       </c>
       <c r="F8" s="14">
-        <v>10009</v>
+        <v>10886</v>
       </c>
       <c r="G8" s="15">
         <f t="shared" si="0"/>
-        <v>25.609000000000002</v>
+        <v>23.315999999999999</v>
       </c>
       <c r="H8" s="15">
         <f t="shared" si="1"/>
-        <v>20.475999999999999</v>
+        <v>21.484000000000002</v>
       </c>
       <c r="I8" s="16">
         <f t="shared" si="2"/>
-        <v>2.5585972624637825</v>
+        <v>2.1418335476759141</v>
       </c>
       <c r="J8" s="17"/>
     </row>
@@ -877,31 +914,31 @@
         <v>16</v>
       </c>
       <c r="B9" s="5">
-        <v>46.69</v>
+        <v>53.65</v>
       </c>
       <c r="C9" s="6">
-        <v>3078</v>
+        <v>3197</v>
       </c>
       <c r="D9" s="7">
-        <v>25584</v>
+        <v>23063</v>
       </c>
       <c r="E9" s="7">
-        <v>23321</v>
+        <v>21642</v>
       </c>
       <c r="F9" s="7">
-        <v>11323</v>
+        <v>11107</v>
       </c>
       <c r="G9" s="8">
         <f t="shared" si="0"/>
-        <v>25.584</v>
+        <v>23.062999999999999</v>
       </c>
       <c r="H9" s="8">
         <f t="shared" si="1"/>
-        <v>23.321000000000002</v>
+        <v>21.641999999999999</v>
       </c>
       <c r="I9" s="9">
         <f t="shared" si="2"/>
-        <v>2.25947187141217</v>
+        <v>2.0764382821644007</v>
       </c>
       <c r="J9" s="10"/>
     </row>
@@ -916,7 +953,7 @@
         <v>3110</v>
       </c>
       <c r="D10" s="14">
-        <v>24835</v>
+        <v>23063</v>
       </c>
       <c r="E10" s="14">
         <v>23063</v>
@@ -926,7 +963,7 @@
       </c>
       <c r="G10" s="15">
         <f t="shared" si="0"/>
-        <v>24.835000000000001</v>
+        <v>23.062999999999999</v>
       </c>
       <c r="H10" s="15">
         <f t="shared" si="1"/>
@@ -934,7 +971,7 @@
       </c>
       <c r="I10" s="16">
         <f t="shared" si="2"/>
-        <v>2.2255578456850973</v>
+        <v>2.066762254682319</v>
       </c>
       <c r="J10" s="17"/>
     </row>
@@ -943,31 +980,31 @@
         <v>18</v>
       </c>
       <c r="B11" s="5">
-        <v>70.47</v>
+        <v>54.2</v>
       </c>
       <c r="C11" s="6">
-        <v>3481</v>
+        <v>2992</v>
       </c>
       <c r="D11" s="7">
-        <v>24724</v>
+        <v>23063</v>
       </c>
       <c r="E11" s="7">
-        <v>21521</v>
+        <v>23063</v>
       </c>
       <c r="F11" s="7">
-        <v>10886</v>
+        <v>11982</v>
       </c>
       <c r="G11" s="8">
         <f t="shared" si="0"/>
-        <v>24.724</v>
+        <v>23.062999999999999</v>
       </c>
       <c r="H11" s="8">
         <f t="shared" si="1"/>
-        <v>21.521000000000001</v>
+        <v>23.062999999999999</v>
       </c>
       <c r="I11" s="9">
         <f t="shared" si="2"/>
-        <v>2.2711739849347787</v>
+        <v>1.9248038724753798</v>
       </c>
       <c r="J11" s="10"/>
     </row>
@@ -976,31 +1013,31 @@
         <v>19</v>
       </c>
       <c r="B12" s="12">
-        <v>263.77999999999997</v>
+        <v>61.56</v>
       </c>
       <c r="C12" s="13">
-        <v>6934</v>
+        <v>3161</v>
       </c>
       <c r="D12" s="14">
-        <v>24642</v>
+        <v>23063</v>
       </c>
       <c r="E12" s="14">
-        <v>19867</v>
+        <v>22217</v>
       </c>
       <c r="F12" s="14">
-        <v>9384</v>
+        <v>11726</v>
       </c>
       <c r="G12" s="15">
         <f t="shared" si="0"/>
-        <v>24.641999999999999</v>
+        <v>23.062999999999999</v>
       </c>
       <c r="H12" s="15">
         <f t="shared" si="1"/>
-        <v>19.867000000000001</v>
+        <v>22.216999999999999</v>
       </c>
       <c r="I12" s="16">
         <f t="shared" si="2"/>
-        <v>2.6259590792838874</v>
+        <v>1.9668258570697594</v>
       </c>
       <c r="J12" s="17"/>
     </row>
@@ -1009,31 +1046,31 @@
         <v>20</v>
       </c>
       <c r="B13" s="5">
-        <v>52.01</v>
+        <v>67.819999999999993</v>
       </c>
       <c r="C13" s="6">
-        <v>3100</v>
+        <v>4140</v>
       </c>
       <c r="D13" s="7">
-        <v>24439</v>
+        <v>21541</v>
       </c>
       <c r="E13" s="7">
-        <v>23234</v>
+        <v>20437</v>
       </c>
       <c r="F13" s="7">
-        <v>10871</v>
+        <v>10009</v>
       </c>
       <c r="G13" s="8">
         <f t="shared" si="0"/>
-        <v>24.439</v>
+        <v>21.541</v>
       </c>
       <c r="H13" s="8">
         <f t="shared" si="1"/>
-        <v>23.234000000000002</v>
+        <v>20.437000000000001</v>
       </c>
       <c r="I13" s="9">
         <f t="shared" si="2"/>
-        <v>2.248091251954742</v>
+        <v>2.1521630532520732</v>
       </c>
       <c r="J13" s="10"/>
     </row>
@@ -1042,31 +1079,31 @@
         <v>21</v>
       </c>
       <c r="B14" s="12">
-        <v>53.65</v>
+        <v>263.77999999999997</v>
       </c>
       <c r="C14" s="13">
-        <v>3197</v>
+        <v>6934</v>
       </c>
       <c r="D14" s="14">
-        <v>24426</v>
+        <v>21515</v>
       </c>
       <c r="E14" s="14">
-        <v>21680</v>
+        <v>19824</v>
       </c>
       <c r="F14" s="14">
-        <v>11107</v>
+        <v>9384</v>
       </c>
       <c r="G14" s="15">
         <f t="shared" si="0"/>
-        <v>24.425999999999998</v>
+        <v>21.515000000000001</v>
       </c>
       <c r="H14" s="15">
         <f t="shared" si="1"/>
-        <v>21.68</v>
+        <v>19.824000000000002</v>
       </c>
       <c r="I14" s="16">
         <f t="shared" si="2"/>
-        <v>2.1991536868641397</v>
+        <v>2.2927323103154307</v>
       </c>
       <c r="J14" s="17"/>
     </row>
@@ -1075,31 +1112,31 @@
         <v>22</v>
       </c>
       <c r="B15" s="5">
-        <v>51.45</v>
+        <v>50.64</v>
       </c>
       <c r="C15" s="6">
-        <v>3530</v>
+        <v>3002</v>
       </c>
       <c r="D15" s="7">
-        <v>21939</v>
+        <v>20762</v>
       </c>
       <c r="E15" s="7">
-        <v>20181</v>
+        <v>19097</v>
       </c>
       <c r="F15" s="7">
-        <v>9210</v>
+        <v>8442</v>
       </c>
       <c r="G15" s="8">
         <f t="shared" si="0"/>
-        <v>21.939</v>
+        <v>20.762</v>
       </c>
       <c r="H15" s="8">
         <f t="shared" si="1"/>
-        <v>20.181000000000001</v>
+        <v>19.097000000000001</v>
       </c>
       <c r="I15" s="9">
         <f t="shared" si="2"/>
-        <v>2.3820846905537461</v>
+        <v>2.4593698175787728</v>
       </c>
       <c r="J15" s="10"/>
     </row>
@@ -1114,25 +1151,25 @@
         <v>3147</v>
       </c>
       <c r="D16" s="14">
-        <v>21740</v>
+        <v>20360</v>
       </c>
       <c r="E16" s="14">
-        <v>20020</v>
+        <v>19963</v>
       </c>
       <c r="F16" s="14">
         <v>8842</v>
       </c>
       <c r="G16" s="15">
         <f t="shared" si="0"/>
-        <v>21.74</v>
+        <v>20.36</v>
       </c>
       <c r="H16" s="15">
         <f t="shared" si="1"/>
-        <v>20.02</v>
+        <v>19.963000000000001</v>
       </c>
       <c r="I16" s="16">
         <f t="shared" si="2"/>
-        <v>2.4587197466636508</v>
+        <v>2.3026464600769057</v>
       </c>
       <c r="J16" s="17"/>
     </row>
@@ -1141,31 +1178,31 @@
         <v>24</v>
       </c>
       <c r="B17" s="5">
-        <v>143</v>
+        <v>63.94</v>
       </c>
       <c r="C17" s="6">
-        <v>5499</v>
+        <v>3736</v>
       </c>
       <c r="D17" s="7">
-        <v>21533</v>
+        <v>20051</v>
       </c>
       <c r="E17" s="7">
-        <v>18280</v>
+        <v>19044</v>
       </c>
       <c r="F17" s="7">
-        <v>8307</v>
+        <v>9056</v>
       </c>
       <c r="G17" s="8">
         <f t="shared" si="0"/>
-        <v>21.533000000000001</v>
+        <v>20.050999999999998</v>
       </c>
       <c r="H17" s="8">
         <f t="shared" si="1"/>
-        <v>18.28</v>
+        <v>19.044</v>
       </c>
       <c r="I17" s="9">
         <f t="shared" si="2"/>
-        <v>2.5921511977850007</v>
+        <v>2.2141121908127208</v>
       </c>
       <c r="J17" s="10"/>
     </row>
@@ -1174,31 +1211,31 @@
         <v>25</v>
       </c>
       <c r="B18" s="12">
-        <v>63.94</v>
+        <v>99.15</v>
       </c>
       <c r="C18" s="13">
-        <v>3736</v>
+        <v>4640</v>
       </c>
       <c r="D18" s="14">
-        <v>21375</v>
+        <v>19372</v>
       </c>
       <c r="E18" s="14">
-        <v>19092</v>
+        <v>18491</v>
       </c>
       <c r="F18" s="14">
-        <v>9056</v>
+        <v>8248</v>
       </c>
       <c r="G18" s="15">
         <f t="shared" si="0"/>
-        <v>21.375</v>
+        <v>19.372</v>
       </c>
       <c r="H18" s="15">
         <f t="shared" si="1"/>
-        <v>19.091999999999999</v>
+        <v>18.491</v>
       </c>
       <c r="I18" s="16">
         <f t="shared" si="2"/>
-        <v>2.3603136042402828</v>
+        <v>2.3486905916585838</v>
       </c>
       <c r="J18" s="17"/>
     </row>
@@ -1207,31 +1244,31 @@
         <v>26</v>
       </c>
       <c r="B19" s="5">
-        <v>14.18</v>
+        <v>96.37</v>
       </c>
       <c r="C19" s="6">
-        <v>1756</v>
+        <v>4536</v>
       </c>
       <c r="D19" s="7">
-        <v>21275</v>
+        <v>19372</v>
       </c>
       <c r="E19" s="7">
-        <v>15931</v>
+        <v>18491</v>
       </c>
       <c r="F19" s="7">
-        <v>7912</v>
+        <v>8256</v>
       </c>
       <c r="G19" s="8">
         <f t="shared" si="0"/>
-        <v>21.274999999999999</v>
+        <v>19.372</v>
       </c>
       <c r="H19" s="8">
         <f t="shared" si="1"/>
-        <v>15.930999999999999</v>
+        <v>18.491</v>
       </c>
       <c r="I19" s="9">
         <f t="shared" si="2"/>
-        <v>2.6889534883720931</v>
+        <v>2.3464147286821704</v>
       </c>
       <c r="J19" s="10"/>
     </row>
@@ -1240,31 +1277,31 @@
         <v>27</v>
       </c>
       <c r="B20" s="12">
-        <v>99.15</v>
+        <v>143</v>
       </c>
       <c r="C20" s="13">
-        <v>4640</v>
+        <v>5499</v>
       </c>
       <c r="D20" s="14">
-        <v>21092</v>
+        <v>19372</v>
       </c>
       <c r="E20" s="14">
-        <v>18515</v>
+        <v>18466</v>
       </c>
       <c r="F20" s="14">
-        <v>8248</v>
+        <v>8307</v>
       </c>
       <c r="G20" s="15">
         <f t="shared" si="0"/>
-        <v>21.091999999999999</v>
+        <v>19.372</v>
       </c>
       <c r="H20" s="15">
         <f t="shared" si="1"/>
-        <v>18.515000000000001</v>
+        <v>18.466000000000001</v>
       </c>
       <c r="I20" s="16">
         <f t="shared" si="2"/>
-        <v>2.5572259941804072</v>
+        <v>2.3320091489105574</v>
       </c>
       <c r="J20" s="17"/>
     </row>
@@ -1273,31 +1310,31 @@
         <v>28</v>
       </c>
       <c r="B21" s="5">
-        <v>96.37</v>
+        <v>43.25</v>
       </c>
       <c r="C21" s="6">
-        <v>4536</v>
+        <v>3108</v>
       </c>
       <c r="D21" s="7">
-        <v>21079</v>
+        <v>19127</v>
       </c>
       <c r="E21" s="7">
-        <v>18515</v>
+        <v>18329</v>
       </c>
       <c r="F21" s="7">
-        <v>8256</v>
+        <v>8461</v>
       </c>
       <c r="G21" s="8">
         <f t="shared" si="0"/>
-        <v>21.079000000000001</v>
+        <v>19.126999999999999</v>
       </c>
       <c r="H21" s="8">
         <f t="shared" si="1"/>
-        <v>18.515000000000001</v>
+        <v>18.329000000000001</v>
       </c>
       <c r="I21" s="9">
         <f t="shared" si="2"/>
-        <v>2.553173449612403</v>
+        <v>2.2606074932041129</v>
       </c>
       <c r="J21" s="10"/>
     </row>
@@ -1306,31 +1343,31 @@
         <v>29</v>
       </c>
       <c r="B22" s="12">
-        <v>50.64</v>
+        <v>54.78</v>
       </c>
       <c r="C22" s="13">
-        <v>3002</v>
+        <v>3399</v>
       </c>
       <c r="D22" s="14">
-        <v>20999</v>
+        <v>19097</v>
       </c>
       <c r="E22" s="14">
-        <v>16635</v>
+        <v>18329</v>
       </c>
       <c r="F22" s="14">
-        <v>8442</v>
+        <v>9205</v>
       </c>
       <c r="G22" s="15">
         <f t="shared" si="0"/>
-        <v>20.998999999999999</v>
+        <v>19.097000000000001</v>
       </c>
       <c r="H22" s="15">
         <f t="shared" si="1"/>
-        <v>16.635000000000002</v>
+        <v>18.329000000000001</v>
       </c>
       <c r="I22" s="16">
         <f t="shared" si="2"/>
-        <v>2.4874437337123902</v>
+        <v>2.0746333514394353</v>
       </c>
       <c r="J22" s="17"/>
     </row>
@@ -1339,31 +1376,31 @@
         <v>30</v>
       </c>
       <c r="B23" s="5">
-        <v>54.78</v>
+        <v>95.86</v>
       </c>
       <c r="C23" s="6">
-        <v>3399</v>
+        <v>4455</v>
       </c>
       <c r="D23" s="7">
-        <v>20405</v>
+        <v>18515</v>
       </c>
       <c r="E23" s="7">
-        <v>18366</v>
+        <v>16914</v>
       </c>
       <c r="F23" s="7">
-        <v>9205</v>
+        <v>7221</v>
       </c>
       <c r="G23" s="8">
         <f t="shared" si="0"/>
-        <v>20.405000000000001</v>
+        <v>18.515000000000001</v>
       </c>
       <c r="H23" s="8">
         <f t="shared" si="1"/>
-        <v>18.366</v>
+        <v>16.914000000000001</v>
       </c>
       <c r="I23" s="9">
         <f t="shared" si="2"/>
-        <v>2.2167300380228139</v>
+        <v>2.5640493006508795</v>
       </c>
       <c r="J23" s="10"/>
     </row>
@@ -1378,25 +1415,25 @@
         <v>5071</v>
       </c>
       <c r="D24" s="14">
-        <v>20081</v>
+        <v>17362</v>
       </c>
       <c r="E24" s="14">
-        <v>16829</v>
+        <v>16756</v>
       </c>
       <c r="F24" s="14">
         <v>9352</v>
       </c>
       <c r="G24" s="15">
         <f t="shared" si="0"/>
-        <v>20.081</v>
+        <v>17.361999999999998</v>
       </c>
       <c r="H24" s="15">
         <f t="shared" si="1"/>
-        <v>16.829000000000001</v>
+        <v>16.756</v>
       </c>
       <c r="I24" s="16">
         <f t="shared" si="2"/>
-        <v>2.1472412318220702</v>
+        <v>1.8565012831479897</v>
       </c>
       <c r="J24" s="17"/>
     </row>
@@ -1405,31 +1442,31 @@
         <v>32</v>
       </c>
       <c r="B25" s="5">
-        <v>95.86</v>
+        <v>114.58</v>
       </c>
       <c r="C25" s="6">
-        <v>4455</v>
+        <v>5085</v>
       </c>
       <c r="D25" s="7">
-        <v>19928</v>
+        <v>17310</v>
       </c>
       <c r="E25" s="7">
-        <v>16953</v>
+        <v>15817</v>
       </c>
       <c r="F25" s="7">
-        <v>7221</v>
+        <v>8501</v>
       </c>
       <c r="G25" s="8">
         <f t="shared" si="0"/>
-        <v>19.928000000000001</v>
+        <v>17.309999999999999</v>
       </c>
       <c r="H25" s="8">
         <f t="shared" si="1"/>
-        <v>16.952999999999999</v>
+        <v>15.817</v>
       </c>
       <c r="I25" s="9">
         <f t="shared" si="2"/>
-        <v>2.7597285694502145</v>
+        <v>2.0362310316433363</v>
       </c>
       <c r="J25" s="10"/>
     </row>
@@ -1438,31 +1475,31 @@
         <v>33</v>
       </c>
       <c r="B26" s="12">
-        <v>43.25</v>
+        <v>73.88</v>
       </c>
       <c r="C26" s="13">
-        <v>3108</v>
+        <v>4134</v>
       </c>
       <c r="D26" s="14">
-        <v>19528</v>
+        <v>17310</v>
       </c>
       <c r="E26" s="14">
-        <v>16655</v>
+        <v>15702</v>
       </c>
       <c r="F26" s="14">
-        <v>8461</v>
+        <v>7712</v>
       </c>
       <c r="G26" s="15">
         <f t="shared" si="0"/>
-        <v>19.527999999999999</v>
+        <v>17.309999999999999</v>
       </c>
       <c r="H26" s="15">
         <f t="shared" si="1"/>
-        <v>16.655000000000001</v>
+        <v>15.702</v>
       </c>
       <c r="I26" s="16">
         <f t="shared" si="2"/>
-        <v>2.3080014182720721</v>
+        <v>2.2445539419087135</v>
       </c>
       <c r="J26" s="17"/>
     </row>
@@ -1471,31 +1508,31 @@
         <v>34</v>
       </c>
       <c r="B27" s="5">
-        <v>114.58</v>
+        <v>148.91</v>
       </c>
       <c r="C27" s="6">
-        <v>5085</v>
+        <v>5858</v>
       </c>
       <c r="D27" s="7">
-        <v>19019</v>
+        <v>17310</v>
       </c>
       <c r="E27" s="7">
-        <v>15835</v>
+        <v>15702</v>
       </c>
       <c r="F27" s="7">
-        <v>8501</v>
+        <v>7712</v>
       </c>
       <c r="G27" s="8">
         <f t="shared" si="0"/>
-        <v>19.018999999999998</v>
+        <v>17.309999999999999</v>
       </c>
       <c r="H27" s="8">
         <f t="shared" si="1"/>
-        <v>15.835000000000001</v>
+        <v>15.702</v>
       </c>
       <c r="I27" s="9">
         <f t="shared" si="2"/>
-        <v>2.2372662039760027</v>
+        <v>2.2445539419087135</v>
       </c>
       <c r="J27" s="10"/>
     </row>
@@ -1504,31 +1541,31 @@
         <v>35</v>
       </c>
       <c r="B28" s="12">
-        <v>108.06</v>
+        <v>264.72000000000003</v>
       </c>
       <c r="C28" s="13">
-        <v>5283</v>
+        <v>6929</v>
       </c>
       <c r="D28" s="14">
-        <v>18650</v>
+        <v>17310</v>
       </c>
       <c r="E28" s="14">
-        <v>15201</v>
+        <v>13787</v>
       </c>
       <c r="F28" s="14">
-        <v>9732</v>
+        <v>6957</v>
       </c>
       <c r="G28" s="15">
         <f t="shared" si="0"/>
-        <v>18.649999999999999</v>
+        <v>17.309999999999999</v>
       </c>
       <c r="H28" s="15">
         <f t="shared" si="1"/>
-        <v>15.201000000000001</v>
+        <v>13.787000000000001</v>
       </c>
       <c r="I28" s="16">
         <f t="shared" si="2"/>
-        <v>1.9163584052609945</v>
+        <v>2.4881414402759812</v>
       </c>
       <c r="J28" s="17"/>
     </row>
@@ -1543,25 +1580,25 @@
         <v>2739</v>
       </c>
       <c r="D29" s="7">
-        <v>17942</v>
+        <v>16982</v>
       </c>
       <c r="E29" s="7">
-        <v>15441</v>
+        <v>16442</v>
       </c>
       <c r="F29" s="7">
         <v>7775</v>
       </c>
       <c r="G29" s="8">
         <f t="shared" si="0"/>
-        <v>17.942</v>
+        <v>16.981999999999999</v>
       </c>
       <c r="H29" s="8">
         <f t="shared" si="1"/>
-        <v>15.441000000000001</v>
+        <v>16.442</v>
       </c>
       <c r="I29" s="9">
         <f t="shared" si="2"/>
-        <v>2.3076527331189709</v>
+        <v>2.1841800643086815</v>
       </c>
       <c r="J29" s="10"/>
     </row>
@@ -1570,31 +1607,31 @@
         <v>37</v>
       </c>
       <c r="B30" s="12">
-        <v>148.91</v>
+        <v>113.04</v>
       </c>
       <c r="C30" s="13">
-        <v>5858</v>
+        <v>5041</v>
       </c>
       <c r="D30" s="14">
-        <v>17938</v>
+        <v>16871</v>
       </c>
       <c r="E30" s="14">
-        <v>14870</v>
+        <v>14208</v>
       </c>
       <c r="F30" s="14">
-        <v>7712</v>
+        <v>8850</v>
       </c>
       <c r="G30" s="15">
         <f t="shared" si="0"/>
-        <v>17.937999999999999</v>
+        <v>16.870999999999999</v>
       </c>
       <c r="H30" s="15">
         <f t="shared" si="1"/>
-        <v>14.87</v>
+        <v>14.208</v>
       </c>
       <c r="I30" s="16">
         <f t="shared" si="2"/>
-        <v>2.3259854771784232</v>
+        <v>1.9063276836158192</v>
       </c>
       <c r="J30" s="17"/>
     </row>
@@ -1603,31 +1640,31 @@
         <v>38</v>
       </c>
       <c r="B31" s="5">
-        <v>73.88</v>
+        <v>108.06</v>
       </c>
       <c r="C31" s="6">
-        <v>4134</v>
+        <v>5283</v>
       </c>
       <c r="D31" s="7">
-        <v>17911</v>
+        <v>16841</v>
       </c>
       <c r="E31" s="7">
-        <v>15728</v>
+        <v>15187</v>
       </c>
       <c r="F31" s="7">
-        <v>7712</v>
+        <v>9732</v>
       </c>
       <c r="G31" s="8">
         <f t="shared" si="0"/>
-        <v>17.911000000000001</v>
+        <v>16.841000000000001</v>
       </c>
       <c r="H31" s="8">
         <f t="shared" si="1"/>
-        <v>15.728</v>
+        <v>15.186999999999999</v>
       </c>
       <c r="I31" s="9">
         <f t="shared" si="2"/>
-        <v>2.322484439834025</v>
+        <v>1.7304767776407728</v>
       </c>
       <c r="J31" s="10"/>
     </row>
@@ -1636,31 +1673,31 @@
         <v>39</v>
       </c>
       <c r="B32" s="12">
-        <v>264.72000000000003</v>
+        <v>14.18</v>
       </c>
       <c r="C32" s="13">
-        <v>6929</v>
+        <v>1756</v>
       </c>
       <c r="D32" s="14">
-        <v>17353</v>
+        <v>16629</v>
       </c>
       <c r="E32" s="14">
-        <v>13853</v>
+        <v>15894</v>
       </c>
       <c r="F32" s="14">
-        <v>6957</v>
+        <v>7912</v>
       </c>
       <c r="G32" s="15">
         <f t="shared" si="0"/>
-        <v>17.353000000000002</v>
+        <v>16.629000000000001</v>
       </c>
       <c r="H32" s="15">
         <f t="shared" si="1"/>
-        <v>13.853</v>
+        <v>15.894</v>
       </c>
       <c r="I32" s="16">
         <f t="shared" si="2"/>
-        <v>2.4943222653442576</v>
+        <v>2.1017441860465116</v>
       </c>
       <c r="J32" s="17"/>
     </row>
@@ -1669,31 +1706,31 @@
         <v>40</v>
       </c>
       <c r="B33" s="5">
-        <v>113.04</v>
+        <v>110.23</v>
       </c>
       <c r="C33" s="6">
-        <v>5041</v>
+        <v>5065</v>
       </c>
       <c r="D33" s="7">
-        <v>17244</v>
+        <v>16426</v>
       </c>
       <c r="E33" s="7">
-        <v>14242</v>
+        <v>14267</v>
       </c>
       <c r="F33" s="7">
-        <v>8850</v>
+        <v>9477</v>
       </c>
       <c r="G33" s="8">
         <f t="shared" si="0"/>
-        <v>17.244</v>
+        <v>16.425999999999998</v>
       </c>
       <c r="H33" s="8">
         <f t="shared" si="1"/>
-        <v>14.242000000000001</v>
+        <v>14.266999999999999</v>
       </c>
       <c r="I33" s="9">
         <f t="shared" si="2"/>
-        <v>1.9484745762711864</v>
+        <v>1.7332489184341036</v>
       </c>
       <c r="J33" s="10"/>
     </row>
@@ -1702,31 +1739,31 @@
         <v>41</v>
       </c>
       <c r="B34" s="12">
-        <v>51.93</v>
+        <v>100.42</v>
       </c>
       <c r="C34" s="13">
-        <v>3411</v>
+        <v>5093</v>
       </c>
       <c r="D34" s="14">
-        <v>17032</v>
+        <v>15892</v>
       </c>
       <c r="E34" s="14">
-        <v>14861</v>
+        <v>14294</v>
       </c>
       <c r="F34" s="14">
-        <v>7991</v>
+        <v>7977</v>
       </c>
       <c r="G34" s="15">
         <f t="shared" si="0"/>
-        <v>17.032</v>
+        <v>15.891999999999999</v>
       </c>
       <c r="H34" s="15">
         <f t="shared" si="1"/>
-        <v>14.861000000000001</v>
+        <v>14.294</v>
       </c>
       <c r="I34" s="16">
         <f t="shared" si="2"/>
-        <v>2.1313978225503694</v>
+        <v>1.9922276545067068</v>
       </c>
       <c r="J34" s="17"/>
     </row>
@@ -1735,31 +1772,31 @@
         <v>42</v>
       </c>
       <c r="B35" s="5">
-        <v>100.42</v>
+        <v>51.93</v>
       </c>
       <c r="C35" s="6">
-        <v>5093</v>
+        <v>3411</v>
       </c>
       <c r="D35" s="7">
-        <v>16586</v>
+        <v>15849</v>
       </c>
       <c r="E35" s="7">
-        <v>13406</v>
+        <v>14818</v>
       </c>
       <c r="F35" s="7">
-        <v>7977</v>
+        <v>7991</v>
       </c>
       <c r="G35" s="8">
         <f t="shared" si="0"/>
-        <v>16.585999999999999</v>
+        <v>15.849</v>
       </c>
       <c r="H35" s="8">
         <f t="shared" si="1"/>
-        <v>13.406000000000001</v>
+        <v>14.818</v>
       </c>
       <c r="I35" s="9">
         <f t="shared" si="2"/>
-        <v>2.0792277798671179</v>
+        <v>1.9833562758102865</v>
       </c>
       <c r="J35" s="10"/>
     </row>
@@ -1774,25 +1811,25 @@
         <v>5134</v>
       </c>
       <c r="D36" s="14">
-        <v>16505</v>
+        <v>14757</v>
       </c>
       <c r="E36" s="14">
-        <v>13811</v>
+        <v>13779</v>
       </c>
       <c r="F36" s="14">
         <v>10367</v>
       </c>
       <c r="G36" s="15">
         <f t="shared" si="0"/>
-        <v>16.504999999999999</v>
+        <v>14.757</v>
       </c>
       <c r="H36" s="15">
         <f t="shared" si="1"/>
-        <v>13.811</v>
+        <v>13.779</v>
       </c>
       <c r="I36" s="16">
         <f t="shared" si="2"/>
-        <v>1.5920709945017846</v>
+        <v>1.4234590527635766</v>
       </c>
       <c r="J36" s="17"/>
     </row>
@@ -1801,31 +1838,31 @@
         <v>44</v>
       </c>
       <c r="B37" s="5">
-        <v>110.23</v>
+        <v>107.45</v>
       </c>
       <c r="C37" s="6">
-        <v>5065</v>
+        <v>5565</v>
       </c>
       <c r="D37" s="7">
-        <v>16444</v>
+        <v>13280</v>
       </c>
       <c r="E37" s="7">
-        <v>12725</v>
+        <v>12164</v>
       </c>
       <c r="F37" s="7">
-        <v>9477</v>
+        <v>7077</v>
       </c>
       <c r="G37" s="8">
         <f t="shared" si="0"/>
-        <v>16.443999999999999</v>
+        <v>13.28</v>
       </c>
       <c r="H37" s="8">
         <f t="shared" si="1"/>
-        <v>12.725</v>
+        <v>12.164</v>
       </c>
       <c r="I37" s="9">
         <f t="shared" si="2"/>
-        <v>1.7351482536667722</v>
+        <v>1.8765013423767134</v>
       </c>
       <c r="J37" s="10"/>
     </row>
@@ -1840,85 +1877,84 @@
         <v>9468</v>
       </c>
       <c r="D38" s="14">
-        <v>15825</v>
+        <v>12672</v>
       </c>
       <c r="E38" s="14">
-        <v>10678</v>
+        <v>10636</v>
       </c>
       <c r="F38" s="14">
         <v>7561</v>
       </c>
       <c r="G38" s="15">
         <f t="shared" si="0"/>
-        <v>15.824999999999999</v>
+        <v>12.672000000000001</v>
       </c>
       <c r="H38" s="15">
         <f t="shared" si="1"/>
-        <v>10.678000000000001</v>
+        <v>10.635999999999999</v>
       </c>
       <c r="I38" s="16">
         <f t="shared" si="2"/>
-        <v>2.0929771194286468</v>
+        <v>1.6759687871974607</v>
       </c>
       <c r="J38" s="17"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="B39" s="5">
-        <v>107.45</v>
-      </c>
-      <c r="C39" s="6">
-        <v>5565</v>
-      </c>
-      <c r="D39" s="7">
-        <v>15610</v>
-      </c>
-      <c r="E39" s="7">
-        <v>12208</v>
-      </c>
-      <c r="F39" s="7">
-        <v>7077</v>
-      </c>
-      <c r="G39" s="8">
-        <f t="shared" si="0"/>
-        <v>15.61</v>
-      </c>
-      <c r="H39" s="8">
-        <f t="shared" si="1"/>
-        <v>12.208</v>
-      </c>
-      <c r="I39" s="9">
-        <f t="shared" si="2"/>
-        <v>2.2057368941641937</v>
-      </c>
-      <c r="J39" s="10"/>
+      <c r="B39" s="19">
+        <v>51.45</v>
+      </c>
+      <c r="C39" s="20">
+        <v>3530</v>
+      </c>
+      <c r="D39" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="E39" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="F39" s="22">
+        <v>9210</v>
+      </c>
+      <c r="G39" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="H39" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="I39" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="J39" s="25" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A41" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="B41" s="19">
+      <c r="A41" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="B41" s="27">
         <f>SUM(B5:B39)</f>
-        <v>3213.16</v>
-      </c>
-      <c r="D41" s="20">
+        <v>3213.1599999999989</v>
+      </c>
+      <c r="D41" s="28">
         <f>MAX(D5:D39)</f>
-        <v>26692</v>
-      </c>
-      <c r="G41" s="21">
+        <v>23878</v>
+      </c>
+      <c r="G41" s="29">
         <f>IFERROR(MAX(G5:G39),"")</f>
-        <v>26.692</v>
-      </c>
-      <c r="I41" s="22">
+        <v>23.878</v>
+      </c>
+      <c r="I41" s="30">
         <f>IFERROR(AVERAGE(I5:I39),"")</f>
-        <v>2.2882355100239358</v>
+        <v>2.0981985652324129</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A42" s="23" t="s">
-        <v>48</v>
+      <c r="A42" s="31" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1936,88 +1972,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
-        <v>49</v>
+      <c r="A1" s="32" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="25" t="s">
-        <v>50</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>51</v>
+      <c r="A3" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" s="34" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="25" t="s">
-        <v>52</v>
-      </c>
-      <c r="B4" s="26" t="s">
-        <v>53</v>
+      <c r="A4" s="33" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="34" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="25" t="s">
-        <v>54</v>
-      </c>
-      <c r="B5" s="26" t="s">
-        <v>55</v>
+      <c r="A5" s="33" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" s="34" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="25" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6" s="26" t="s">
-        <v>57</v>
+      <c r="A6" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" s="34" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="B7" s="26" t="s">
-        <v>59</v>
+      <c r="A7" s="33" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" s="34" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="25" t="s">
-        <v>60</v>
-      </c>
-      <c r="B8" s="26" t="s">
-        <v>61</v>
+      <c r="A8" s="33" t="s">
+        <v>63</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="25" t="s">
-        <v>62</v>
-      </c>
-      <c r="B9" s="26" t="s">
-        <v>63</v>
+      <c r="A9" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="B9" s="34" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B10" s="26" t="s">
-        <v>65</v>
+      <c r="A10" s="33" t="s">
+        <v>67</v>
+      </c>
+      <c r="B10" s="34" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="B11" s="26" t="s">
-        <v>67</v>
+      <c r="A11" s="33" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="34" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="25" t="s">
-        <v>68</v>
-      </c>
-      <c r="B12" s="26" t="s">
-        <v>69</v>
+      <c r="A12" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" s="34" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Simulador de estrada fictícia; tabela de pendências; cor de P.Pedra
Novo: com um talhão selecionado, "Simular nova estrada" desenha uma linha
no mapa e recalcula MÁX/MÍN localmente no navegador (Dijkstra em JS, mesma
regra do pipeline: só estrada desenhada, sem divisa) — não grava nada em
lugar nenhum, é só pra explorar "e se desenhasse aqui?" antes de desenhar
de verdade na bancada.

Recalculado com as duas correções do pipeline desta sessão (estradas que se
cruzam agora ligam entre si; sede conecta a cada pedaço de estrada
separado, não só aos 15 mais próximos no total) — sem acesso caiu de 60
para 7 talhões.

Menu Pendências agora tem duas tabelas: talhões sem estrada mapeada (por
talhão, não só contagem por fazenda) e talhões com contorno sobreposto no
KML (achado numa conferência manual — contorno antigo de antes da
subdivisão, precisa corrigir no Google Earth).

Cor de Ponte de Pedra trocada de verde pra vermelho — verde não destacava
contra a lavoura, também verde.
</commit_message>
<xml_diff>
--- a/FAZENDA_JAVA_distancias.xlsx
+++ b/FAZENDA_JAVA_distancias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\talhao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BBA2AD1-FAC8-43C4-849A-42B1D6480D99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06BEC0FB-46A2-4187-A43F-BE65DFB6B447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,106 +72,106 @@
     <t>Observação</t>
   </si>
   <si>
+    <t>T-11A</t>
+  </si>
+  <si>
+    <t>T-13C</t>
+  </si>
+  <si>
+    <t>T-13B</t>
+  </si>
+  <si>
     <t>T-11B</t>
   </si>
   <si>
+    <t>T-13D</t>
+  </si>
+  <si>
+    <t>T-11D</t>
+  </si>
+  <si>
+    <t>T-13A</t>
+  </si>
+  <si>
     <t>T-11C</t>
   </si>
   <si>
-    <t>T-11A</t>
-  </si>
-  <si>
-    <t>T-11D</t>
-  </si>
-  <si>
-    <t>T-13A</t>
-  </si>
-  <si>
-    <t>T-13B</t>
-  </si>
-  <si>
-    <t>T-13C</t>
-  </si>
-  <si>
-    <t>T-13D</t>
-  </si>
-  <si>
     <t>T-10A</t>
   </si>
   <si>
     <t>T-12A</t>
   </si>
   <si>
+    <t>T-14A</t>
+  </si>
+  <si>
+    <t>T-14D</t>
+  </si>
+  <si>
+    <t>T-07C</t>
+  </si>
+  <si>
+    <t>T-07D</t>
+  </si>
+  <si>
+    <t>T-15C</t>
+  </si>
+  <si>
+    <t>T-07B</t>
+  </si>
+  <si>
     <t>T-07A</t>
   </si>
   <si>
+    <t>T-05</t>
+  </si>
+  <si>
+    <t>T-01C</t>
+  </si>
+  <si>
+    <t>T-06B</t>
+  </si>
+  <si>
+    <t>T-06D</t>
+  </si>
+  <si>
+    <t>T-06E</t>
+  </si>
+  <si>
     <t>T-09A</t>
   </si>
   <si>
-    <t>T-07B</t>
-  </si>
-  <si>
-    <t>T-14A</t>
-  </si>
-  <si>
-    <t>T-14D</t>
+    <t>T-06C</t>
+  </si>
+  <si>
+    <t>T-03B</t>
+  </si>
+  <si>
+    <t>T-03A</t>
+  </si>
+  <si>
+    <t>T-08A</t>
+  </si>
+  <si>
+    <t>T-01</t>
+  </si>
+  <si>
+    <t>T-04A</t>
+  </si>
+  <si>
+    <t>T-04B</t>
+  </si>
+  <si>
+    <t>T-01A</t>
+  </si>
+  <si>
+    <t>T-04</t>
+  </si>
+  <si>
+    <t>T-02</t>
   </si>
   <si>
     <t>T-15B</t>
-  </si>
-  <si>
-    <t>T-07D</t>
-  </si>
-  <si>
-    <t>T-07C</t>
-  </si>
-  <si>
-    <t>T-15C</t>
-  </si>
-  <si>
-    <t>T-05</t>
-  </si>
-  <si>
-    <t>T-01C</t>
-  </si>
-  <si>
-    <t>T-06B</t>
-  </si>
-  <si>
-    <t>T-06D</t>
-  </si>
-  <si>
-    <t>T-06E</t>
-  </si>
-  <si>
-    <t>T-06C</t>
-  </si>
-  <si>
-    <t>T-03B</t>
-  </si>
-  <si>
-    <t>T-03A</t>
-  </si>
-  <si>
-    <t>T-08A</t>
-  </si>
-  <si>
-    <t>T-01</t>
-  </si>
-  <si>
-    <t>T-04A</t>
-  </si>
-  <si>
-    <t>T-04B</t>
-  </si>
-  <si>
-    <t>T-01A</t>
-  </si>
-  <si>
-    <t>T-04</t>
-  </si>
-  <si>
-    <t>T-02</t>
   </si>
   <si>
     <t>T-09B</t>
@@ -782,31 +782,31 @@
         <v>12</v>
       </c>
       <c r="B5" s="5">
-        <v>46.69</v>
+        <v>61.24</v>
       </c>
       <c r="C5" s="6">
-        <v>3078</v>
+        <v>3271</v>
       </c>
       <c r="D5" s="7">
-        <v>23878</v>
+        <v>26425</v>
       </c>
       <c r="E5" s="7">
-        <v>23285</v>
+        <v>25324</v>
       </c>
       <c r="F5" s="7">
-        <v>11323</v>
+        <v>11475</v>
       </c>
       <c r="G5" s="8">
         <f t="shared" ref="G5:G38" si="0">D5/1000</f>
-        <v>23.878</v>
+        <v>26.425000000000001</v>
       </c>
       <c r="H5" s="8">
         <f t="shared" ref="H5:H38" si="1">E5/1000</f>
-        <v>23.285</v>
+        <v>25.324000000000002</v>
       </c>
       <c r="I5" s="9">
         <f t="shared" ref="I5:I38" si="2">IFERROR(D5/F5,"")</f>
-        <v>2.1088050869910799</v>
+        <v>2.3028322440087146</v>
       </c>
       <c r="J5" s="10"/>
     </row>
@@ -815,31 +815,31 @@
         <v>13</v>
       </c>
       <c r="B6" s="12">
-        <v>52.01</v>
+        <v>54.2</v>
       </c>
       <c r="C6" s="13">
-        <v>3100</v>
+        <v>2992</v>
       </c>
       <c r="D6" s="14">
-        <v>23878</v>
+        <v>26143</v>
       </c>
       <c r="E6" s="14">
-        <v>23285</v>
+        <v>24523</v>
       </c>
       <c r="F6" s="14">
-        <v>10871</v>
+        <v>11982</v>
       </c>
       <c r="G6" s="15">
         <f t="shared" si="0"/>
-        <v>23.878</v>
+        <v>26.143000000000001</v>
       </c>
       <c r="H6" s="15">
         <f t="shared" si="1"/>
-        <v>23.285</v>
+        <v>24.523</v>
       </c>
       <c r="I6" s="16">
         <f t="shared" si="2"/>
-        <v>2.1964860638395733</v>
+        <v>2.1818561175095978</v>
       </c>
       <c r="J6" s="17"/>
     </row>
@@ -848,31 +848,31 @@
         <v>14</v>
       </c>
       <c r="B7" s="5">
-        <v>61.24</v>
+        <v>58.52</v>
       </c>
       <c r="C7" s="6">
-        <v>3271</v>
+        <v>3110</v>
       </c>
       <c r="D7" s="7">
-        <v>23316</v>
+        <v>24573</v>
       </c>
       <c r="E7" s="7">
-        <v>22217</v>
+        <v>23560</v>
       </c>
       <c r="F7" s="7">
-        <v>11475</v>
+        <v>11159</v>
       </c>
       <c r="G7" s="8">
         <f t="shared" si="0"/>
-        <v>23.315999999999999</v>
+        <v>24.573</v>
       </c>
       <c r="H7" s="8">
         <f t="shared" si="1"/>
-        <v>22.216999999999999</v>
+        <v>23.56</v>
       </c>
       <c r="I7" s="9">
         <f t="shared" si="2"/>
-        <v>2.0318954248366015</v>
+        <v>2.2020790393404428</v>
       </c>
       <c r="J7" s="10"/>
     </row>
@@ -881,31 +881,31 @@
         <v>15</v>
       </c>
       <c r="B8" s="12">
-        <v>70.47</v>
+        <v>46.69</v>
       </c>
       <c r="C8" s="13">
-        <v>3481</v>
+        <v>3078</v>
       </c>
       <c r="D8" s="14">
-        <v>23316</v>
+        <v>23903</v>
       </c>
       <c r="E8" s="14">
-        <v>21484</v>
+        <v>23311</v>
       </c>
       <c r="F8" s="14">
-        <v>10886</v>
+        <v>11323</v>
       </c>
       <c r="G8" s="15">
         <f t="shared" si="0"/>
-        <v>23.315999999999999</v>
+        <v>23.902999999999999</v>
       </c>
       <c r="H8" s="15">
         <f t="shared" si="1"/>
-        <v>21.484000000000002</v>
+        <v>23.311</v>
       </c>
       <c r="I8" s="16">
         <f t="shared" si="2"/>
-        <v>2.1418335476759141</v>
+        <v>2.1110129824251525</v>
       </c>
       <c r="J8" s="17"/>
     </row>
@@ -914,31 +914,31 @@
         <v>16</v>
       </c>
       <c r="B9" s="5">
-        <v>53.65</v>
+        <v>61.56</v>
       </c>
       <c r="C9" s="6">
-        <v>3197</v>
+        <v>3161</v>
       </c>
       <c r="D9" s="7">
-        <v>23063</v>
+        <v>23559</v>
       </c>
       <c r="E9" s="7">
-        <v>21642</v>
+        <v>22243</v>
       </c>
       <c r="F9" s="7">
-        <v>11107</v>
+        <v>11726</v>
       </c>
       <c r="G9" s="8">
         <f t="shared" si="0"/>
-        <v>23.062999999999999</v>
+        <v>23.559000000000001</v>
       </c>
       <c r="H9" s="8">
         <f t="shared" si="1"/>
-        <v>21.641999999999999</v>
+        <v>22.242999999999999</v>
       </c>
       <c r="I9" s="9">
         <f t="shared" si="2"/>
-        <v>2.0764382821644007</v>
+        <v>2.0091250213201435</v>
       </c>
       <c r="J9" s="10"/>
     </row>
@@ -947,31 +947,31 @@
         <v>17</v>
       </c>
       <c r="B10" s="12">
-        <v>58.52</v>
+        <v>70.47</v>
       </c>
       <c r="C10" s="13">
-        <v>3110</v>
+        <v>3481</v>
       </c>
       <c r="D10" s="14">
-        <v>23063</v>
+        <v>23341</v>
       </c>
       <c r="E10" s="14">
-        <v>23063</v>
+        <v>21510</v>
       </c>
       <c r="F10" s="14">
-        <v>11159</v>
+        <v>10886</v>
       </c>
       <c r="G10" s="15">
         <f t="shared" si="0"/>
-        <v>23.062999999999999</v>
+        <v>23.341000000000001</v>
       </c>
       <c r="H10" s="15">
         <f t="shared" si="1"/>
-        <v>23.062999999999999</v>
+        <v>21.51</v>
       </c>
       <c r="I10" s="16">
         <f t="shared" si="2"/>
-        <v>2.066762254682319</v>
+        <v>2.1441300753261068</v>
       </c>
       <c r="J10" s="17"/>
     </row>
@@ -980,31 +980,31 @@
         <v>18</v>
       </c>
       <c r="B11" s="5">
-        <v>54.2</v>
+        <v>53.65</v>
       </c>
       <c r="C11" s="6">
-        <v>2992</v>
+        <v>3197</v>
       </c>
       <c r="D11" s="7">
-        <v>23063</v>
+        <v>23161</v>
       </c>
       <c r="E11" s="7">
-        <v>23063</v>
+        <v>21667</v>
       </c>
       <c r="F11" s="7">
-        <v>11982</v>
+        <v>11107</v>
       </c>
       <c r="G11" s="8">
         <f t="shared" si="0"/>
-        <v>23.062999999999999</v>
+        <v>23.161000000000001</v>
       </c>
       <c r="H11" s="8">
         <f t="shared" si="1"/>
-        <v>23.062999999999999</v>
+        <v>21.667000000000002</v>
       </c>
       <c r="I11" s="9">
         <f t="shared" si="2"/>
-        <v>1.9248038724753798</v>
+        <v>2.0852615467723057</v>
       </c>
       <c r="J11" s="10"/>
     </row>
@@ -1013,31 +1013,31 @@
         <v>19</v>
       </c>
       <c r="B12" s="12">
-        <v>61.56</v>
+        <v>52.01</v>
       </c>
       <c r="C12" s="13">
-        <v>3161</v>
+        <v>3100</v>
       </c>
       <c r="D12" s="14">
-        <v>23063</v>
+        <v>23158</v>
       </c>
       <c r="E12" s="14">
-        <v>22217</v>
+        <v>22257</v>
       </c>
       <c r="F12" s="14">
-        <v>11726</v>
+        <v>10871</v>
       </c>
       <c r="G12" s="15">
         <f t="shared" si="0"/>
-        <v>23.062999999999999</v>
+        <v>23.158000000000001</v>
       </c>
       <c r="H12" s="15">
         <f t="shared" si="1"/>
-        <v>22.216999999999999</v>
+        <v>22.257000000000001</v>
       </c>
       <c r="I12" s="16">
         <f t="shared" si="2"/>
-        <v>1.9668258570697594</v>
+        <v>2.1302548063655595</v>
       </c>
       <c r="J12" s="17"/>
     </row>
@@ -1052,25 +1052,25 @@
         <v>4140</v>
       </c>
       <c r="D13" s="7">
-        <v>21541</v>
+        <v>22301</v>
       </c>
       <c r="E13" s="7">
-        <v>20437</v>
+        <v>20463</v>
       </c>
       <c r="F13" s="7">
         <v>10009</v>
       </c>
       <c r="G13" s="8">
         <f t="shared" si="0"/>
-        <v>21.541</v>
+        <v>22.300999999999998</v>
       </c>
       <c r="H13" s="8">
         <f t="shared" si="1"/>
-        <v>20.437000000000001</v>
+        <v>20.463000000000001</v>
       </c>
       <c r="I13" s="9">
         <f t="shared" si="2"/>
-        <v>2.1521630532520732</v>
+        <v>2.2280947147567192</v>
       </c>
       <c r="J13" s="10"/>
     </row>
@@ -1085,25 +1085,25 @@
         <v>6934</v>
       </c>
       <c r="D14" s="14">
-        <v>21515</v>
+        <v>21540</v>
       </c>
       <c r="E14" s="14">
-        <v>19824</v>
+        <v>19850</v>
       </c>
       <c r="F14" s="14">
         <v>9384</v>
       </c>
       <c r="G14" s="15">
         <f t="shared" si="0"/>
-        <v>21.515000000000001</v>
+        <v>21.54</v>
       </c>
       <c r="H14" s="15">
         <f t="shared" si="1"/>
-        <v>19.824000000000002</v>
+        <v>19.850000000000001</v>
       </c>
       <c r="I14" s="16">
         <f t="shared" si="2"/>
-        <v>2.2927323103154307</v>
+        <v>2.2953964194373402</v>
       </c>
       <c r="J14" s="17"/>
     </row>
@@ -1112,31 +1112,31 @@
         <v>22</v>
       </c>
       <c r="B15" s="5">
-        <v>50.64</v>
+        <v>99.15</v>
       </c>
       <c r="C15" s="6">
-        <v>3002</v>
+        <v>4640</v>
       </c>
       <c r="D15" s="7">
-        <v>20762</v>
+        <v>19397</v>
       </c>
       <c r="E15" s="7">
-        <v>19097</v>
+        <v>18517</v>
       </c>
       <c r="F15" s="7">
-        <v>8442</v>
+        <v>8248</v>
       </c>
       <c r="G15" s="8">
         <f t="shared" si="0"/>
-        <v>20.762</v>
+        <v>19.396999999999998</v>
       </c>
       <c r="H15" s="8">
         <f t="shared" si="1"/>
-        <v>19.097000000000001</v>
+        <v>18.516999999999999</v>
       </c>
       <c r="I15" s="9">
         <f t="shared" si="2"/>
-        <v>2.4593698175787728</v>
+        <v>2.3517216294859358</v>
       </c>
       <c r="J15" s="10"/>
     </row>
@@ -1145,31 +1145,31 @@
         <v>23</v>
       </c>
       <c r="B16" s="12">
-        <v>51.15</v>
+        <v>96.37</v>
       </c>
       <c r="C16" s="13">
-        <v>3147</v>
+        <v>4536</v>
       </c>
       <c r="D16" s="14">
-        <v>20360</v>
+        <v>19397</v>
       </c>
       <c r="E16" s="14">
-        <v>19963</v>
+        <v>18517</v>
       </c>
       <c r="F16" s="14">
-        <v>8842</v>
+        <v>8256</v>
       </c>
       <c r="G16" s="15">
         <f t="shared" si="0"/>
-        <v>20.36</v>
+        <v>19.396999999999998</v>
       </c>
       <c r="H16" s="15">
         <f t="shared" si="1"/>
-        <v>19.963000000000001</v>
+        <v>18.516999999999999</v>
       </c>
       <c r="I16" s="16">
         <f t="shared" si="2"/>
-        <v>2.3026464600769057</v>
+        <v>2.3494428294573644</v>
       </c>
       <c r="J16" s="17"/>
     </row>
@@ -1178,31 +1178,31 @@
         <v>24</v>
       </c>
       <c r="B17" s="5">
-        <v>63.94</v>
+        <v>54.78</v>
       </c>
       <c r="C17" s="6">
-        <v>3736</v>
+        <v>3399</v>
       </c>
       <c r="D17" s="7">
-        <v>20051</v>
+        <v>18624</v>
       </c>
       <c r="E17" s="7">
-        <v>19044</v>
+        <v>18131</v>
       </c>
       <c r="F17" s="7">
-        <v>9056</v>
+        <v>9205</v>
       </c>
       <c r="G17" s="8">
         <f t="shared" si="0"/>
-        <v>20.050999999999998</v>
+        <v>18.623999999999999</v>
       </c>
       <c r="H17" s="8">
         <f t="shared" si="1"/>
-        <v>19.044</v>
+        <v>18.131</v>
       </c>
       <c r="I17" s="9">
         <f t="shared" si="2"/>
-        <v>2.2141121908127208</v>
+        <v>2.0232482346550786</v>
       </c>
       <c r="J17" s="10"/>
     </row>
@@ -1211,31 +1211,31 @@
         <v>25</v>
       </c>
       <c r="B18" s="12">
-        <v>99.15</v>
+        <v>43.25</v>
       </c>
       <c r="C18" s="13">
-        <v>4640</v>
+        <v>3108</v>
       </c>
       <c r="D18" s="14">
-        <v>19372</v>
+        <v>18624</v>
       </c>
       <c r="E18" s="14">
-        <v>18491</v>
+        <v>18102</v>
       </c>
       <c r="F18" s="14">
-        <v>8248</v>
+        <v>8461</v>
       </c>
       <c r="G18" s="15">
         <f t="shared" si="0"/>
-        <v>19.372</v>
+        <v>18.623999999999999</v>
       </c>
       <c r="H18" s="15">
         <f t="shared" si="1"/>
-        <v>18.491</v>
+        <v>18.102</v>
       </c>
       <c r="I18" s="16">
         <f t="shared" si="2"/>
-        <v>2.3486905916585838</v>
+        <v>2.2011582555253515</v>
       </c>
       <c r="J18" s="17"/>
     </row>
@@ -1244,31 +1244,31 @@
         <v>26</v>
       </c>
       <c r="B19" s="5">
-        <v>96.37</v>
+        <v>95.86</v>
       </c>
       <c r="C19" s="6">
-        <v>4536</v>
+        <v>4455</v>
       </c>
       <c r="D19" s="7">
-        <v>19372</v>
+        <v>18541</v>
       </c>
       <c r="E19" s="7">
-        <v>18491</v>
+        <v>16940</v>
       </c>
       <c r="F19" s="7">
-        <v>8256</v>
+        <v>7221</v>
       </c>
       <c r="G19" s="8">
         <f t="shared" si="0"/>
-        <v>19.372</v>
+        <v>18.541</v>
       </c>
       <c r="H19" s="8">
         <f t="shared" si="1"/>
-        <v>18.491</v>
+        <v>16.940000000000001</v>
       </c>
       <c r="I19" s="9">
         <f t="shared" si="2"/>
-        <v>2.3464147286821704</v>
+        <v>2.5676499099847665</v>
       </c>
       <c r="J19" s="10"/>
     </row>
@@ -1277,31 +1277,31 @@
         <v>27</v>
       </c>
       <c r="B20" s="12">
-        <v>143</v>
+        <v>63.94</v>
       </c>
       <c r="C20" s="13">
-        <v>5499</v>
+        <v>3736</v>
       </c>
       <c r="D20" s="14">
-        <v>19372</v>
+        <v>18184</v>
       </c>
       <c r="E20" s="14">
-        <v>18466</v>
+        <v>17178</v>
       </c>
       <c r="F20" s="14">
-        <v>8307</v>
+        <v>9056</v>
       </c>
       <c r="G20" s="15">
         <f t="shared" si="0"/>
-        <v>19.372</v>
+        <v>18.184000000000001</v>
       </c>
       <c r="H20" s="15">
         <f t="shared" si="1"/>
-        <v>18.466000000000001</v>
+        <v>17.178000000000001</v>
       </c>
       <c r="I20" s="16">
         <f t="shared" si="2"/>
-        <v>2.3320091489105574</v>
+        <v>2.0079505300353357</v>
       </c>
       <c r="J20" s="17"/>
     </row>
@@ -1310,31 +1310,31 @@
         <v>28</v>
       </c>
       <c r="B21" s="5">
-        <v>43.25</v>
+        <v>50.64</v>
       </c>
       <c r="C21" s="6">
-        <v>3108</v>
+        <v>3002</v>
       </c>
       <c r="D21" s="7">
-        <v>19127</v>
+        <v>18131</v>
       </c>
       <c r="E21" s="7">
-        <v>18329</v>
+        <v>16467</v>
       </c>
       <c r="F21" s="7">
-        <v>8461</v>
+        <v>8442</v>
       </c>
       <c r="G21" s="8">
         <f t="shared" si="0"/>
-        <v>19.126999999999999</v>
+        <v>18.131</v>
       </c>
       <c r="H21" s="8">
         <f t="shared" si="1"/>
-        <v>18.329000000000001</v>
+        <v>16.466999999999999</v>
       </c>
       <c r="I21" s="9">
         <f t="shared" si="2"/>
-        <v>2.2606074932041129</v>
+        <v>2.1477138118929164</v>
       </c>
       <c r="J21" s="10"/>
     </row>
@@ -1343,31 +1343,31 @@
         <v>29</v>
       </c>
       <c r="B22" s="12">
-        <v>54.78</v>
+        <v>114.01</v>
       </c>
       <c r="C22" s="13">
-        <v>3399</v>
+        <v>5071</v>
       </c>
       <c r="D22" s="14">
-        <v>19097</v>
+        <v>17388</v>
       </c>
       <c r="E22" s="14">
-        <v>18329</v>
+        <v>16782</v>
       </c>
       <c r="F22" s="14">
-        <v>9205</v>
+        <v>9352</v>
       </c>
       <c r="G22" s="15">
         <f t="shared" si="0"/>
-        <v>19.097000000000001</v>
+        <v>17.388000000000002</v>
       </c>
       <c r="H22" s="15">
         <f t="shared" si="1"/>
-        <v>18.329000000000001</v>
+        <v>16.782</v>
       </c>
       <c r="I22" s="16">
         <f t="shared" si="2"/>
-        <v>2.0746333514394353</v>
+        <v>1.8592814371257484</v>
       </c>
       <c r="J22" s="17"/>
     </row>
@@ -1376,31 +1376,31 @@
         <v>30</v>
       </c>
       <c r="B23" s="5">
-        <v>95.86</v>
+        <v>114.58</v>
       </c>
       <c r="C23" s="6">
-        <v>4455</v>
+        <v>5085</v>
       </c>
       <c r="D23" s="7">
-        <v>18515</v>
+        <v>17322</v>
       </c>
       <c r="E23" s="7">
-        <v>16914</v>
+        <v>15789</v>
       </c>
       <c r="F23" s="7">
-        <v>7221</v>
+        <v>8501</v>
       </c>
       <c r="G23" s="8">
         <f t="shared" si="0"/>
-        <v>18.515000000000001</v>
+        <v>17.321999999999999</v>
       </c>
       <c r="H23" s="8">
         <f t="shared" si="1"/>
-        <v>16.914000000000001</v>
+        <v>15.789</v>
       </c>
       <c r="I23" s="9">
         <f t="shared" si="2"/>
-        <v>2.5640493006508795</v>
+        <v>2.0376426302787909</v>
       </c>
       <c r="J23" s="10"/>
     </row>
@@ -1409,31 +1409,31 @@
         <v>31</v>
       </c>
       <c r="B24" s="12">
-        <v>114.01</v>
+        <v>73.88</v>
       </c>
       <c r="C24" s="13">
-        <v>5071</v>
+        <v>4134</v>
       </c>
       <c r="D24" s="14">
-        <v>17362</v>
+        <v>17322</v>
       </c>
       <c r="E24" s="14">
-        <v>16756</v>
+        <v>15727</v>
       </c>
       <c r="F24" s="14">
-        <v>9352</v>
+        <v>7712</v>
       </c>
       <c r="G24" s="15">
         <f t="shared" si="0"/>
-        <v>17.361999999999998</v>
+        <v>17.321999999999999</v>
       </c>
       <c r="H24" s="15">
         <f t="shared" si="1"/>
-        <v>16.756</v>
+        <v>15.727</v>
       </c>
       <c r="I24" s="16">
         <f t="shared" si="2"/>
-        <v>1.8565012831479897</v>
+        <v>2.2461099585062239</v>
       </c>
       <c r="J24" s="17"/>
     </row>
@@ -1442,31 +1442,31 @@
         <v>32</v>
       </c>
       <c r="B25" s="5">
-        <v>114.58</v>
+        <v>148.91</v>
       </c>
       <c r="C25" s="6">
-        <v>5085</v>
+        <v>5858</v>
       </c>
       <c r="D25" s="7">
-        <v>17310</v>
+        <v>17322</v>
       </c>
       <c r="E25" s="7">
-        <v>15817</v>
+        <v>15727</v>
       </c>
       <c r="F25" s="7">
-        <v>8501</v>
+        <v>7712</v>
       </c>
       <c r="G25" s="8">
         <f t="shared" si="0"/>
-        <v>17.309999999999999</v>
+        <v>17.321999999999999</v>
       </c>
       <c r="H25" s="8">
         <f t="shared" si="1"/>
-        <v>15.817</v>
+        <v>15.727</v>
       </c>
       <c r="I25" s="9">
         <f t="shared" si="2"/>
-        <v>2.0362310316433363</v>
+        <v>2.2461099585062239</v>
       </c>
       <c r="J25" s="10"/>
     </row>
@@ -1475,31 +1475,31 @@
         <v>33</v>
       </c>
       <c r="B26" s="12">
-        <v>73.88</v>
+        <v>264.72000000000003</v>
       </c>
       <c r="C26" s="13">
-        <v>4134</v>
+        <v>6929</v>
       </c>
       <c r="D26" s="14">
-        <v>17310</v>
+        <v>17322</v>
       </c>
       <c r="E26" s="14">
-        <v>15702</v>
+        <v>13813</v>
       </c>
       <c r="F26" s="14">
-        <v>7712</v>
+        <v>6957</v>
       </c>
       <c r="G26" s="15">
         <f t="shared" si="0"/>
-        <v>17.309999999999999</v>
+        <v>17.321999999999999</v>
       </c>
       <c r="H26" s="15">
         <f t="shared" si="1"/>
-        <v>15.702</v>
+        <v>13.813000000000001</v>
       </c>
       <c r="I26" s="16">
         <f t="shared" si="2"/>
-        <v>2.2445539419087135</v>
+        <v>2.4898663216903838</v>
       </c>
       <c r="J26" s="17"/>
     </row>
@@ -1508,31 +1508,31 @@
         <v>34</v>
       </c>
       <c r="B27" s="5">
-        <v>148.91</v>
+        <v>51.15</v>
       </c>
       <c r="C27" s="6">
-        <v>5858</v>
+        <v>3147</v>
       </c>
       <c r="D27" s="7">
-        <v>17310</v>
+        <v>17266</v>
       </c>
       <c r="E27" s="7">
-        <v>15702</v>
+        <v>16869</v>
       </c>
       <c r="F27" s="7">
-        <v>7712</v>
+        <v>8842</v>
       </c>
       <c r="G27" s="8">
         <f t="shared" si="0"/>
-        <v>17.309999999999999</v>
+        <v>17.265999999999998</v>
       </c>
       <c r="H27" s="8">
         <f t="shared" si="1"/>
-        <v>15.702</v>
+        <v>16.869</v>
       </c>
       <c r="I27" s="9">
         <f t="shared" si="2"/>
-        <v>2.2445539419087135</v>
+        <v>1.9527256276860439</v>
       </c>
       <c r="J27" s="10"/>
     </row>
@@ -1541,31 +1541,31 @@
         <v>35</v>
       </c>
       <c r="B28" s="12">
-        <v>264.72000000000003</v>
+        <v>31.74</v>
       </c>
       <c r="C28" s="13">
-        <v>6929</v>
+        <v>2739</v>
       </c>
       <c r="D28" s="14">
-        <v>17310</v>
+        <v>16983</v>
       </c>
       <c r="E28" s="14">
-        <v>13787</v>
+        <v>16443</v>
       </c>
       <c r="F28" s="14">
-        <v>6957</v>
+        <v>7775</v>
       </c>
       <c r="G28" s="15">
         <f t="shared" si="0"/>
-        <v>17.309999999999999</v>
+        <v>16.983000000000001</v>
       </c>
       <c r="H28" s="15">
         <f t="shared" si="1"/>
-        <v>13.787000000000001</v>
+        <v>16.443000000000001</v>
       </c>
       <c r="I28" s="16">
         <f t="shared" si="2"/>
-        <v>2.4881414402759812</v>
+        <v>2.1843086816720256</v>
       </c>
       <c r="J28" s="17"/>
     </row>
@@ -1574,31 +1574,31 @@
         <v>36</v>
       </c>
       <c r="B29" s="5">
-        <v>31.74</v>
+        <v>113.04</v>
       </c>
       <c r="C29" s="6">
-        <v>2739</v>
+        <v>5041</v>
       </c>
       <c r="D29" s="7">
-        <v>16982</v>
+        <v>16896</v>
       </c>
       <c r="E29" s="7">
-        <v>16442</v>
+        <v>14233</v>
       </c>
       <c r="F29" s="7">
-        <v>7775</v>
+        <v>8850</v>
       </c>
       <c r="G29" s="8">
         <f t="shared" si="0"/>
-        <v>16.981999999999999</v>
+        <v>16.896000000000001</v>
       </c>
       <c r="H29" s="8">
         <f t="shared" si="1"/>
-        <v>16.442</v>
+        <v>14.233000000000001</v>
       </c>
       <c r="I29" s="9">
         <f t="shared" si="2"/>
-        <v>2.1841800643086815</v>
+        <v>1.9091525423728815</v>
       </c>
       <c r="J29" s="10"/>
     </row>
@@ -1607,31 +1607,31 @@
         <v>37</v>
       </c>
       <c r="B30" s="12">
-        <v>113.04</v>
+        <v>108.06</v>
       </c>
       <c r="C30" s="13">
-        <v>5041</v>
+        <v>5283</v>
       </c>
       <c r="D30" s="14">
-        <v>16871</v>
+        <v>16867</v>
       </c>
       <c r="E30" s="14">
-        <v>14208</v>
+        <v>15212</v>
       </c>
       <c r="F30" s="14">
-        <v>8850</v>
+        <v>9732</v>
       </c>
       <c r="G30" s="15">
         <f t="shared" si="0"/>
-        <v>16.870999999999999</v>
+        <v>16.867000000000001</v>
       </c>
       <c r="H30" s="15">
         <f t="shared" si="1"/>
-        <v>14.208</v>
+        <v>15.212</v>
       </c>
       <c r="I30" s="16">
         <f t="shared" si="2"/>
-        <v>1.9063276836158192</v>
+        <v>1.73314837648993</v>
       </c>
       <c r="J30" s="17"/>
     </row>
@@ -1640,31 +1640,31 @@
         <v>38</v>
       </c>
       <c r="B31" s="5">
-        <v>108.06</v>
+        <v>14.18</v>
       </c>
       <c r="C31" s="6">
-        <v>5283</v>
+        <v>1756</v>
       </c>
       <c r="D31" s="7">
-        <v>16841</v>
+        <v>16654</v>
       </c>
       <c r="E31" s="7">
-        <v>15187</v>
+        <v>15919</v>
       </c>
       <c r="F31" s="7">
-        <v>9732</v>
+        <v>7912</v>
       </c>
       <c r="G31" s="8">
         <f t="shared" si="0"/>
-        <v>16.841000000000001</v>
+        <v>16.654</v>
       </c>
       <c r="H31" s="8">
         <f t="shared" si="1"/>
-        <v>15.186999999999999</v>
+        <v>15.919</v>
       </c>
       <c r="I31" s="9">
         <f t="shared" si="2"/>
-        <v>1.7304767776407728</v>
+        <v>2.1049039433771486</v>
       </c>
       <c r="J31" s="10"/>
     </row>
@@ -1673,31 +1673,31 @@
         <v>39</v>
       </c>
       <c r="B32" s="12">
-        <v>14.18</v>
+        <v>110.23</v>
       </c>
       <c r="C32" s="13">
-        <v>1756</v>
+        <v>5065</v>
       </c>
       <c r="D32" s="14">
-        <v>16629</v>
+        <v>16452</v>
       </c>
       <c r="E32" s="14">
-        <v>15894</v>
+        <v>12673</v>
       </c>
       <c r="F32" s="14">
-        <v>7912</v>
+        <v>9477</v>
       </c>
       <c r="G32" s="15">
         <f t="shared" si="0"/>
-        <v>16.629000000000001</v>
+        <v>16.452000000000002</v>
       </c>
       <c r="H32" s="15">
         <f t="shared" si="1"/>
-        <v>15.894</v>
+        <v>12.673</v>
       </c>
       <c r="I32" s="16">
         <f t="shared" si="2"/>
-        <v>2.1017441860465116</v>
+        <v>1.7359924026590694</v>
       </c>
       <c r="J32" s="17"/>
     </row>
@@ -1706,31 +1706,31 @@
         <v>40</v>
       </c>
       <c r="B33" s="5">
-        <v>110.23</v>
+        <v>100.42</v>
       </c>
       <c r="C33" s="6">
-        <v>5065</v>
+        <v>5093</v>
       </c>
       <c r="D33" s="7">
-        <v>16426</v>
+        <v>15893</v>
       </c>
       <c r="E33" s="7">
-        <v>14267</v>
+        <v>14319</v>
       </c>
       <c r="F33" s="7">
-        <v>9477</v>
+        <v>7977</v>
       </c>
       <c r="G33" s="8">
         <f t="shared" si="0"/>
-        <v>16.425999999999998</v>
+        <v>15.893000000000001</v>
       </c>
       <c r="H33" s="8">
         <f t="shared" si="1"/>
-        <v>14.266999999999999</v>
+        <v>14.319000000000001</v>
       </c>
       <c r="I33" s="9">
         <f t="shared" si="2"/>
-        <v>1.7332489184341036</v>
+        <v>1.992353014917889</v>
       </c>
       <c r="J33" s="10"/>
     </row>
@@ -1739,31 +1739,31 @@
         <v>41</v>
       </c>
       <c r="B34" s="12">
-        <v>100.42</v>
+        <v>51.93</v>
       </c>
       <c r="C34" s="13">
-        <v>5093</v>
+        <v>3411</v>
       </c>
       <c r="D34" s="14">
-        <v>15892</v>
+        <v>15893</v>
       </c>
       <c r="E34" s="14">
-        <v>14294</v>
+        <v>14843</v>
       </c>
       <c r="F34" s="14">
-        <v>7977</v>
+        <v>7991</v>
       </c>
       <c r="G34" s="15">
         <f t="shared" si="0"/>
-        <v>15.891999999999999</v>
+        <v>15.893000000000001</v>
       </c>
       <c r="H34" s="15">
         <f t="shared" si="1"/>
-        <v>14.294</v>
+        <v>14.843</v>
       </c>
       <c r="I34" s="16">
         <f t="shared" si="2"/>
-        <v>1.9922276545067068</v>
+        <v>1.988862470279064</v>
       </c>
       <c r="J34" s="17"/>
     </row>
@@ -1772,31 +1772,31 @@
         <v>42</v>
       </c>
       <c r="B35" s="5">
-        <v>51.93</v>
+        <v>109.74</v>
       </c>
       <c r="C35" s="6">
-        <v>3411</v>
+        <v>5134</v>
       </c>
       <c r="D35" s="7">
-        <v>15849</v>
+        <v>14709</v>
       </c>
       <c r="E35" s="7">
-        <v>14818</v>
+        <v>13784</v>
       </c>
       <c r="F35" s="7">
-        <v>7991</v>
+        <v>10367</v>
       </c>
       <c r="G35" s="8">
         <f t="shared" si="0"/>
-        <v>15.849</v>
+        <v>14.709</v>
       </c>
       <c r="H35" s="8">
         <f t="shared" si="1"/>
-        <v>14.818</v>
+        <v>13.784000000000001</v>
       </c>
       <c r="I35" s="9">
         <f t="shared" si="2"/>
-        <v>1.9833562758102865</v>
+        <v>1.4188289765602393</v>
       </c>
       <c r="J35" s="10"/>
     </row>
@@ -1805,31 +1805,31 @@
         <v>43</v>
       </c>
       <c r="B36" s="12">
-        <v>109.74</v>
+        <v>107.45</v>
       </c>
       <c r="C36" s="13">
-        <v>5134</v>
+        <v>5565</v>
       </c>
       <c r="D36" s="14">
-        <v>14757</v>
+        <v>13305</v>
       </c>
       <c r="E36" s="14">
-        <v>13779</v>
+        <v>12189</v>
       </c>
       <c r="F36" s="14">
-        <v>10367</v>
+        <v>7077</v>
       </c>
       <c r="G36" s="15">
         <f t="shared" si="0"/>
-        <v>14.757</v>
+        <v>13.305</v>
       </c>
       <c r="H36" s="15">
         <f t="shared" si="1"/>
-        <v>13.779</v>
+        <v>12.189</v>
       </c>
       <c r="I36" s="16">
         <f t="shared" si="2"/>
-        <v>1.4234590527635766</v>
+        <v>1.8800339126748622</v>
       </c>
       <c r="J36" s="17"/>
     </row>
@@ -1838,31 +1838,31 @@
         <v>44</v>
       </c>
       <c r="B37" s="5">
-        <v>107.45</v>
+        <v>210.74</v>
       </c>
       <c r="C37" s="6">
-        <v>5565</v>
+        <v>9468</v>
       </c>
       <c r="D37" s="7">
-        <v>13280</v>
+        <v>12697</v>
       </c>
       <c r="E37" s="7">
-        <v>12164</v>
+        <v>10661</v>
       </c>
       <c r="F37" s="7">
-        <v>7077</v>
+        <v>7561</v>
       </c>
       <c r="G37" s="8">
         <f t="shared" si="0"/>
-        <v>13.28</v>
+        <v>12.696999999999999</v>
       </c>
       <c r="H37" s="8">
         <f t="shared" si="1"/>
-        <v>12.164</v>
+        <v>10.661</v>
       </c>
       <c r="I37" s="9">
         <f t="shared" si="2"/>
-        <v>1.8765013423767134</v>
+        <v>1.6792752281444254</v>
       </c>
       <c r="J37" s="10"/>
     </row>
@@ -1871,31 +1871,31 @@
         <v>45</v>
       </c>
       <c r="B38" s="12">
-        <v>210.74</v>
+        <v>143</v>
       </c>
       <c r="C38" s="13">
-        <v>9468</v>
+        <v>5499</v>
       </c>
       <c r="D38" s="14">
-        <v>12672</v>
+        <v>9711</v>
       </c>
       <c r="E38" s="14">
-        <v>10636</v>
+        <v>8841</v>
       </c>
       <c r="F38" s="14">
-        <v>7561</v>
+        <v>8307</v>
       </c>
       <c r="G38" s="15">
         <f t="shared" si="0"/>
-        <v>12.672000000000001</v>
+        <v>9.7110000000000003</v>
       </c>
       <c r="H38" s="15">
         <f t="shared" si="1"/>
-        <v>10.635999999999999</v>
+        <v>8.8409999999999993</v>
       </c>
       <c r="I38" s="16">
         <f t="shared" si="2"/>
-        <v>1.6759687871974607</v>
+        <v>1.1690140845070423</v>
       </c>
       <c r="J38" s="17"/>
     </row>
@@ -1941,15 +1941,15 @@
       </c>
       <c r="D41" s="28">
         <f>MAX(D5:D39)</f>
-        <v>23878</v>
+        <v>26425</v>
       </c>
       <c r="G41" s="29">
         <f>IFERROR(MAX(G5:G39),"")</f>
-        <v>23.878</v>
+        <v>26.425000000000001</v>
       </c>
       <c r="I41" s="30">
         <f>IFERROR(AVERAGE(I5:I39),"")</f>
-        <v>2.0981985652324129</v>
+        <v>2.057839345169024</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
T-09B (Java) sai de "sem acesso" via ponto de exceção confirmado
Mesmo mecanismo já usado em T-05D/T-CON/T-06C (Tucano): usuário identificou
na imagem de satélite que o acesso real de T-09B começa no cruzamento entre
T-07A/T-07B/T-09A, a menos de 1m de uma estrada já digitalizada. Distância
agora é 14,71 km até a sede do Tucano (Java entrega lá), fator 1,60 — em
linha com os talhões vizinhos.

Cache-busting do dados_mapa.js.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FAZENDA_JAVA_distancias.xlsx
+++ b/FAZENDA_JAVA_distancias.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\talhao\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\talhoes-distancias\saidas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{822337A6-3571-4972-ADAE-0EB8A85E8243}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79AF115C-0828-4C2A-A595-8DFDDB60E21A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2232" yWindow="2232" windowWidth="14100" windowHeight="9792" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Distâncias" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
   <si>
     <t>FAZENDA JAVA — distância dos talhões até a sede</t>
   </si>
@@ -144,6 +144,9 @@
     <t>T-09A</t>
   </si>
   <si>
+    <t>T-09B</t>
+  </si>
+  <si>
     <t>T-01A</t>
   </si>
   <si>
@@ -172,18 +175,6 @@
   </si>
   <si>
     <t>T-04</t>
-  </si>
-  <si>
-    <t>T-09B</t>
-  </si>
-  <si>
-    <t>sem acesso</t>
-  </si>
-  <si>
-    <t>—</t>
-  </si>
-  <si>
-    <t>sem estrada até este talhão</t>
   </si>
   <si>
     <t>TOTAL / MÁXIMO</t>
@@ -262,7 +253,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -308,17 +299,6 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FFC00000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="9"/>
-      <color rgb="FFC00000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF808080"/>
@@ -330,7 +310,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -345,11 +325,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -374,7 +349,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -395,25 +370,13 @@
     <xf numFmtId="4" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -797,15 +760,15 @@
         <v>11475</v>
       </c>
       <c r="G5" s="8">
-        <f t="shared" ref="G5:G38" si="0">D5/1000</f>
+        <f t="shared" ref="G5:G39" si="0">D5/1000</f>
         <v>23.838000000000001</v>
       </c>
       <c r="H5" s="8">
-        <f t="shared" ref="H5:H38" si="1">E5/1000</f>
+        <f t="shared" ref="H5:H39" si="1">E5/1000</f>
         <v>22.736999999999998</v>
       </c>
       <c r="I5" s="9">
-        <f t="shared" ref="I5:I38" si="2">IFERROR(D5/F5,"")</f>
+        <f t="shared" ref="I5:I39" si="2">IFERROR(D5/F5,"")</f>
         <v>2.0773856209150328</v>
       </c>
       <c r="J5" s="10"/>
@@ -1574,31 +1537,31 @@
         <v>36</v>
       </c>
       <c r="B29" s="5">
-        <v>109.74</v>
+        <v>51.45</v>
       </c>
       <c r="C29" s="6">
-        <v>5134</v>
+        <v>3530</v>
       </c>
       <c r="D29" s="7">
-        <v>14708</v>
+        <v>14709</v>
       </c>
       <c r="E29" s="7">
-        <v>13783</v>
+        <v>14709</v>
       </c>
       <c r="F29" s="7">
-        <v>10367</v>
+        <v>9210</v>
       </c>
       <c r="G29" s="8">
         <f t="shared" si="0"/>
-        <v>14.708</v>
+        <v>14.709</v>
       </c>
       <c r="H29" s="8">
         <f t="shared" si="1"/>
-        <v>13.782999999999999</v>
+        <v>14.709</v>
       </c>
       <c r="I29" s="9">
         <f t="shared" si="2"/>
-        <v>1.4187325166393363</v>
+        <v>1.5970684039087948</v>
       </c>
       <c r="J29" s="10"/>
     </row>
@@ -1607,31 +1570,31 @@
         <v>37</v>
       </c>
       <c r="B30" s="12">
-        <v>108.06</v>
+        <v>109.74</v>
       </c>
       <c r="C30" s="13">
-        <v>5283</v>
+        <v>5134</v>
       </c>
       <c r="D30" s="14">
-        <v>14601</v>
+        <v>14708</v>
       </c>
       <c r="E30" s="14">
-        <v>13332</v>
+        <v>13783</v>
       </c>
       <c r="F30" s="14">
-        <v>9732</v>
+        <v>10367</v>
       </c>
       <c r="G30" s="15">
         <f t="shared" si="0"/>
-        <v>14.601000000000001</v>
+        <v>14.708</v>
       </c>
       <c r="H30" s="15">
         <f t="shared" si="1"/>
-        <v>13.332000000000001</v>
+        <v>13.782999999999999</v>
       </c>
       <c r="I30" s="16">
         <f t="shared" si="2"/>
-        <v>1.500308261405672</v>
+        <v>1.4187325166393363</v>
       </c>
       <c r="J30" s="17"/>
     </row>
@@ -1640,19 +1603,19 @@
         <v>38</v>
       </c>
       <c r="B31" s="5">
-        <v>113.04</v>
+        <v>108.06</v>
       </c>
       <c r="C31" s="6">
-        <v>5041</v>
+        <v>5283</v>
       </c>
       <c r="D31" s="7">
         <v>14601</v>
       </c>
       <c r="E31" s="7">
-        <v>12353</v>
+        <v>13332</v>
       </c>
       <c r="F31" s="7">
-        <v>8850</v>
+        <v>9732</v>
       </c>
       <c r="G31" s="8">
         <f t="shared" si="0"/>
@@ -1660,11 +1623,11 @@
       </c>
       <c r="H31" s="8">
         <f t="shared" si="1"/>
-        <v>12.353</v>
+        <v>13.332000000000001</v>
       </c>
       <c r="I31" s="9">
         <f t="shared" si="2"/>
-        <v>1.6498305084745764</v>
+        <v>1.500308261405672</v>
       </c>
       <c r="J31" s="10"/>
     </row>
@@ -1673,31 +1636,31 @@
         <v>39</v>
       </c>
       <c r="B32" s="12">
-        <v>110.23</v>
+        <v>113.04</v>
       </c>
       <c r="C32" s="13">
-        <v>5065</v>
+        <v>5041</v>
       </c>
       <c r="D32" s="14">
-        <v>14572</v>
+        <v>14601</v>
       </c>
       <c r="E32" s="14">
-        <v>12412</v>
+        <v>12353</v>
       </c>
       <c r="F32" s="14">
-        <v>9477</v>
+        <v>8850</v>
       </c>
       <c r="G32" s="15">
         <f t="shared" si="0"/>
-        <v>14.571999999999999</v>
+        <v>14.601000000000001</v>
       </c>
       <c r="H32" s="15">
         <f t="shared" si="1"/>
-        <v>12.412000000000001</v>
+        <v>12.353</v>
       </c>
       <c r="I32" s="16">
         <f t="shared" si="2"/>
-        <v>1.5376173894692413</v>
+        <v>1.6498305084745764</v>
       </c>
       <c r="J32" s="17"/>
     </row>
@@ -1706,31 +1669,31 @@
         <v>40</v>
       </c>
       <c r="B33" s="5">
-        <v>31.74</v>
+        <v>110.23</v>
       </c>
       <c r="C33" s="6">
-        <v>2739</v>
+        <v>5065</v>
       </c>
       <c r="D33" s="7">
-        <v>14463</v>
+        <v>14572</v>
       </c>
       <c r="E33" s="7">
-        <v>13923</v>
+        <v>12412</v>
       </c>
       <c r="F33" s="7">
-        <v>7775</v>
+        <v>9477</v>
       </c>
       <c r="G33" s="8">
         <f t="shared" si="0"/>
-        <v>14.462999999999999</v>
+        <v>14.571999999999999</v>
       </c>
       <c r="H33" s="8">
         <f t="shared" si="1"/>
-        <v>13.923</v>
+        <v>12.412000000000001</v>
       </c>
       <c r="I33" s="9">
         <f t="shared" si="2"/>
-        <v>1.8601929260450161</v>
+        <v>1.5376173894692413</v>
       </c>
       <c r="J33" s="10"/>
     </row>
@@ -1739,31 +1702,31 @@
         <v>41</v>
       </c>
       <c r="B34" s="12">
-        <v>14.18</v>
+        <v>31.74</v>
       </c>
       <c r="C34" s="13">
-        <v>1756</v>
+        <v>2739</v>
       </c>
       <c r="D34" s="14">
-        <v>14134</v>
+        <v>14463</v>
       </c>
       <c r="E34" s="14">
-        <v>13399</v>
+        <v>13923</v>
       </c>
       <c r="F34" s="14">
-        <v>7912</v>
+        <v>7775</v>
       </c>
       <c r="G34" s="15">
         <f t="shared" si="0"/>
-        <v>14.134</v>
+        <v>14.462999999999999</v>
       </c>
       <c r="H34" s="15">
         <f t="shared" si="1"/>
-        <v>13.398999999999999</v>
+        <v>13.923</v>
       </c>
       <c r="I34" s="16">
         <f t="shared" si="2"/>
-        <v>1.7864004044489383</v>
+        <v>1.8601929260450161</v>
       </c>
       <c r="J34" s="17"/>
     </row>
@@ -1772,31 +1735,31 @@
         <v>42</v>
       </c>
       <c r="B35" s="5">
-        <v>100.42</v>
+        <v>14.18</v>
       </c>
       <c r="C35" s="6">
-        <v>5093</v>
+        <v>1756</v>
       </c>
       <c r="D35" s="7">
-        <v>13645</v>
+        <v>14134</v>
       </c>
       <c r="E35" s="7">
-        <v>12352</v>
+        <v>13399</v>
       </c>
       <c r="F35" s="7">
-        <v>7977</v>
+        <v>7912</v>
       </c>
       <c r="G35" s="8">
         <f t="shared" si="0"/>
-        <v>13.645</v>
+        <v>14.134</v>
       </c>
       <c r="H35" s="8">
         <f t="shared" si="1"/>
-        <v>12.352</v>
+        <v>13.398999999999999</v>
       </c>
       <c r="I35" s="9">
         <f t="shared" si="2"/>
-        <v>1.7105428105804188</v>
+        <v>1.7864004044489383</v>
       </c>
       <c r="J35" s="10"/>
     </row>
@@ -1805,19 +1768,19 @@
         <v>43</v>
       </c>
       <c r="B36" s="12">
-        <v>51.93</v>
+        <v>100.42</v>
       </c>
       <c r="C36" s="13">
-        <v>3411</v>
+        <v>5093</v>
       </c>
       <c r="D36" s="14">
         <v>13645</v>
       </c>
       <c r="E36" s="14">
-        <v>12323</v>
+        <v>12352</v>
       </c>
       <c r="F36" s="14">
-        <v>7991</v>
+        <v>7977</v>
       </c>
       <c r="G36" s="15">
         <f t="shared" si="0"/>
@@ -1825,11 +1788,11 @@
       </c>
       <c r="H36" s="15">
         <f t="shared" si="1"/>
-        <v>12.323</v>
+        <v>12.352</v>
       </c>
       <c r="I36" s="16">
         <f t="shared" si="2"/>
-        <v>1.7075459892378926</v>
+        <v>1.7105428105804188</v>
       </c>
       <c r="J36" s="17"/>
     </row>
@@ -1838,31 +1801,31 @@
         <v>44</v>
       </c>
       <c r="B37" s="5">
-        <v>210.74</v>
+        <v>51.93</v>
       </c>
       <c r="C37" s="6">
-        <v>9468</v>
+        <v>3411</v>
       </c>
       <c r="D37" s="7">
-        <v>12696</v>
+        <v>13645</v>
       </c>
       <c r="E37" s="7">
-        <v>10412</v>
+        <v>12323</v>
       </c>
       <c r="F37" s="7">
-        <v>7561</v>
+        <v>7991</v>
       </c>
       <c r="G37" s="8">
         <f t="shared" si="0"/>
-        <v>12.696</v>
+        <v>13.645</v>
       </c>
       <c r="H37" s="8">
         <f t="shared" si="1"/>
-        <v>10.412000000000001</v>
+        <v>12.323</v>
       </c>
       <c r="I37" s="9">
         <f t="shared" si="2"/>
-        <v>1.6791429705065468</v>
+        <v>1.7075459892378926</v>
       </c>
       <c r="J37" s="10"/>
     </row>
@@ -1871,90 +1834,91 @@
         <v>45</v>
       </c>
       <c r="B38" s="12">
+        <v>210.74</v>
+      </c>
+      <c r="C38" s="13">
+        <v>9468</v>
+      </c>
+      <c r="D38" s="14">
+        <v>12696</v>
+      </c>
+      <c r="E38" s="14">
+        <v>10412</v>
+      </c>
+      <c r="F38" s="14">
+        <v>7561</v>
+      </c>
+      <c r="G38" s="15">
+        <f t="shared" si="0"/>
+        <v>12.696</v>
+      </c>
+      <c r="H38" s="15">
+        <f t="shared" si="1"/>
+        <v>10.412000000000001</v>
+      </c>
+      <c r="I38" s="16">
+        <f t="shared" si="2"/>
+        <v>1.6791429705065468</v>
+      </c>
+      <c r="J38" s="17"/>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A39" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B39" s="5">
         <v>107.45</v>
       </c>
-      <c r="C38" s="13">
+      <c r="C39" s="6">
         <v>5565</v>
       </c>
-      <c r="D38" s="14">
+      <c r="D39" s="7">
         <v>11425</v>
       </c>
-      <c r="E38" s="14">
+      <c r="E39" s="7">
         <v>10040</v>
       </c>
-      <c r="F38" s="14">
+      <c r="F39" s="7">
         <v>7077</v>
       </c>
-      <c r="G38" s="15">
+      <c r="G39" s="8">
         <f t="shared" si="0"/>
         <v>11.425000000000001</v>
       </c>
-      <c r="H38" s="15">
+      <c r="H39" s="8">
         <f t="shared" si="1"/>
         <v>10.039999999999999</v>
       </c>
-      <c r="I38" s="16">
+      <c r="I39" s="9">
         <f t="shared" si="2"/>
         <v>1.6143846262540624</v>
       </c>
-      <c r="J38" s="17"/>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A39" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="B39" s="19">
-        <v>51.45</v>
-      </c>
-      <c r="C39" s="20">
-        <v>3530</v>
-      </c>
-      <c r="D39" s="21" t="s">
+      <c r="J39" s="10"/>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A41" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="E39" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="F39" s="22">
-        <v>9210</v>
-      </c>
-      <c r="G39" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="H39" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="I39" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="J39" s="25" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A41" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="B41" s="27">
+      <c r="B41" s="19">
         <f>SUM(B5:B39)</f>
         <v>3213.1599999999989</v>
       </c>
-      <c r="D41" s="28">
+      <c r="D41" s="20">
         <f>MAX(D5:D39)</f>
         <v>23838</v>
       </c>
-      <c r="G41" s="29">
+      <c r="G41" s="21">
         <f>IFERROR(MAX(G5:G39),"")</f>
         <v>23.838000000000001</v>
       </c>
-      <c r="I41" s="30">
+      <c r="I41" s="22">
         <f>IFERROR(AVERAGE(I5:I39),"")</f>
-        <v>1.8399301915377113</v>
+        <v>1.8329912833197421</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A42" s="31" t="s">
-        <v>51</v>
+      <c r="A42" s="23" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1972,88 +1936,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="24" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="26" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="25" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="33" t="s">
+      <c r="B4" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="B3" s="34" t="s">
+    </row>
+    <row r="5" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="25" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="33" t="s">
+      <c r="B5" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="B4" s="34" t="s">
+    </row>
+    <row r="6" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="25" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="33" t="s">
+      <c r="B6" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="B5" s="34" t="s">
+    </row>
+    <row r="7" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="25" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="33" t="s">
+      <c r="B7" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="B6" s="34" t="s">
+    </row>
+    <row r="8" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="25" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="33" t="s">
+      <c r="B8" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="B7" s="34" t="s">
+    </row>
+    <row r="9" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="25" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="33" t="s">
+      <c r="B9" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="B8" s="34" t="s">
+    </row>
+    <row r="10" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="25" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="33" t="s">
+      <c r="B10" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="B9" s="34" t="s">
+    </row>
+    <row r="11" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="25" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="33" t="s">
+      <c r="B11" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="B10" s="34" t="s">
+    </row>
+    <row r="12" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="25" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="33" t="s">
+      <c r="B12" s="26" t="s">
         <v>69</v>
-      </c>
-      <c r="B11" s="34" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="33" t="s">
-        <v>71</v>
-      </c>
-      <c r="B12" s="34" t="s">
-        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>